<commit_message>
feat(improv): regenerate Set 01 & Set 02 high-relevance vocab hints, upgrade excel parser with flexible headers, and optimize stage contrast
</commit_message>
<xml_diff>
--- a/public/data/Improv_Set_01_Wandering_Souls.xlsx
+++ b/public/data/Improv_Set_01_Wandering_Souls.xlsx
@@ -397,174 +397,72 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R61"/>
+  <dimension ref="A1:R63"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
+        <v>Set 01 • Wandering Souls (Airport &amp; Travel Reflex)</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>60 progressive deduction items for travel, airport mishaps, and casual spoken reactions based on Level B Day 2.</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
         <v>Session</v>
       </c>
-      <c r="B1" t="str">
+      <c r="B3" t="str">
         <v>Item</v>
       </c>
-      <c r="C1" t="str">
+      <c r="C3" t="str">
         <v>hc-total</v>
       </c>
-      <c r="D1" t="str">
+      <c r="D3" t="str">
         <v>hint-1</v>
       </c>
-      <c r="E1" t="str">
+      <c r="E3" t="str">
+        <v>hint-2</v>
+      </c>
+      <c r="F3" t="str">
+        <v>hint-3</v>
+      </c>
+      <c r="G3" t="str">
+        <v>hint-4</v>
+      </c>
+      <c r="H3" t="str">
+        <v>hint-5</v>
+      </c>
+      <c r="I3" t="str">
         <v>hint-1-translation</v>
       </c>
-      <c r="F1" t="str">
+      <c r="J3" t="str">
+        <v>hint-2-translation</v>
+      </c>
+      <c r="K3" t="str">
+        <v>hint-3-translation</v>
+      </c>
+      <c r="L3" t="str">
+        <v>hint-4-translation</v>
+      </c>
+      <c r="M3" t="str">
+        <v>hint-5-translation</v>
+      </c>
+      <c r="N3" t="str">
         <v>hint-1-type / function</v>
       </c>
-      <c r="G1" t="str">
-        <v>hint-2</v>
-      </c>
-      <c r="H1" t="str">
-        <v>hint-2-translation</v>
-      </c>
-      <c r="I1" t="str">
+      <c r="O3" t="str">
         <v>hint-2-type / function</v>
       </c>
-      <c r="J1" t="str">
-        <v>hint-3</v>
-      </c>
-      <c r="K1" t="str">
-        <v>hint-3-translation</v>
-      </c>
-      <c r="L1" t="str">
+      <c r="P3" t="str">
         <v>hint-3-type / function</v>
       </c>
-      <c r="M1" t="str">
-        <v>hint-4</v>
-      </c>
-      <c r="N1" t="str">
-        <v>hint-4-translation</v>
-      </c>
-      <c r="O1" t="str">
+      <c r="Q3" t="str">
         <v>hint-4-type / function</v>
       </c>
-      <c r="P1" t="str">
-        <v>hint-5</v>
-      </c>
-      <c r="Q1" t="str">
-        <v>hint-5-translation</v>
-      </c>
-      <c r="R1" t="str">
+      <c r="R3" t="str">
         <v>hint-5-type / function</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2">
-        <v>1</v>
-      </c>
-      <c r="C2">
-        <v>2</v>
-      </c>
-      <c r="D2" t="str">
-        <v>customs officer</v>
-      </c>
-      <c r="E2" t="str">
-        <v>nhân viên hải quan</v>
-      </c>
-      <c r="F2" t="str">
-        <v>Keyword</v>
-      </c>
-      <c r="G2" t="str">
-        <v>asked for my passport</v>
-      </c>
-      <c r="H2" t="str">
-        <v>đã yêu cầu xem hộ chiếu</v>
-      </c>
-      <c r="I2" t="str">
-        <v>Ending</v>
-      </c>
-      <c r="J2" t="str">
-        <v/>
-      </c>
-      <c r="K2" t="str">
-        <v/>
-      </c>
-      <c r="L2" t="str">
-        <v/>
-      </c>
-      <c r="M2" t="str">
-        <v/>
-      </c>
-      <c r="N2" t="str">
-        <v/>
-      </c>
-      <c r="O2" t="str">
-        <v/>
-      </c>
-      <c r="P2" t="str">
-        <v/>
-      </c>
-      <c r="Q2" t="str">
-        <v/>
-      </c>
-      <c r="R2" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3">
-        <v>1</v>
-      </c>
-      <c r="B3">
-        <v>2</v>
-      </c>
-      <c r="C3">
-        <v>2</v>
-      </c>
-      <c r="D3" t="str">
-        <v>boarding pass</v>
-      </c>
-      <c r="E3" t="str">
-        <v>thẻ lên máy bay</v>
-      </c>
-      <c r="F3" t="str">
-        <v>Keyword</v>
-      </c>
-      <c r="G3" t="str">
-        <v>handed to the agent</v>
-      </c>
-      <c r="H3" t="str">
-        <v>đã đưa cho nhân viên</v>
-      </c>
-      <c r="I3" t="str">
-        <v>Ending</v>
-      </c>
-      <c r="J3" t="str">
-        <v/>
-      </c>
-      <c r="K3" t="str">
-        <v/>
-      </c>
-      <c r="L3" t="str">
-        <v/>
-      </c>
-      <c r="M3" t="str">
-        <v/>
-      </c>
-      <c r="N3" t="str">
-        <v/>
-      </c>
-      <c r="O3" t="str">
-        <v/>
-      </c>
-      <c r="P3" t="str">
-        <v/>
-      </c>
-      <c r="Q3" t="str">
-        <v/>
-      </c>
-      <c r="R3" t="str">
-        <v/>
       </c>
     </row>
     <row r="4">
@@ -572,31 +470,31 @@
         <v>1</v>
       </c>
       <c r="B4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C4">
         <v>2</v>
       </c>
       <c r="D4" t="str">
-        <v>loose change</v>
+        <v>boarding pass</v>
       </c>
       <c r="E4" t="str">
-        <v>tiền lẻ</v>
+        <v>lost</v>
       </c>
       <c r="F4" t="str">
-        <v>Keyword</v>
+        <v/>
       </c>
       <c r="G4" t="str">
-        <v>left in front pocket</v>
+        <v/>
       </c>
       <c r="H4" t="str">
-        <v>còn sót trong túi trước</v>
+        <v/>
       </c>
       <c r="I4" t="str">
-        <v>Ending</v>
+        <v>thẻ lên máy bay</v>
       </c>
       <c r="J4" t="str">
-        <v/>
+        <v>làm mất</v>
       </c>
       <c r="K4" t="str">
         <v/>
@@ -608,10 +506,10 @@
         <v/>
       </c>
       <c r="N4" t="str">
-        <v/>
+        <v>Danh từ · Keyword</v>
       </c>
       <c r="O4" t="str">
-        <v/>
+        <v>Động từ · Ending</v>
       </c>
       <c r="P4" t="str">
         <v/>
@@ -628,31 +526,31 @@
         <v>1</v>
       </c>
       <c r="B5">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C5">
         <v>2</v>
       </c>
       <c r="D5" t="str">
-        <v>sleeping bag</v>
+        <v>loose change</v>
       </c>
       <c r="E5" t="str">
-        <v>túi ngủ du lịch</v>
+        <v>front pocket</v>
       </c>
       <c r="F5" t="str">
-        <v>Keyword</v>
+        <v/>
       </c>
       <c r="G5" t="str">
-        <v>rolled up neatly</v>
+        <v/>
       </c>
       <c r="H5" t="str">
-        <v>được cuộn gọn gàng</v>
+        <v/>
       </c>
       <c r="I5" t="str">
-        <v>Ending</v>
+        <v>tiền lẻ</v>
       </c>
       <c r="J5" t="str">
-        <v/>
+        <v>túi trước</v>
       </c>
       <c r="K5" t="str">
         <v/>
@@ -664,10 +562,10 @@
         <v/>
       </c>
       <c r="N5" t="str">
-        <v/>
+        <v>Danh từ · Keyword</v>
       </c>
       <c r="O5" t="str">
-        <v/>
+        <v>Danh từ · Ending</v>
       </c>
       <c r="P5" t="str">
         <v/>
@@ -684,7 +582,7 @@
         <v>1</v>
       </c>
       <c r="B6">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C6">
         <v>2</v>
@@ -693,22 +591,22 @@
         <v>luggage cart</v>
       </c>
       <c r="E6" t="str">
+        <v>heavy</v>
+      </c>
+      <c r="F6" t="str">
+        <v/>
+      </c>
+      <c r="G6" t="str">
+        <v/>
+      </c>
+      <c r="H6" t="str">
+        <v/>
+      </c>
+      <c r="I6" t="str">
         <v>xe đẩy hành lý</v>
       </c>
-      <c r="F6" t="str">
-        <v>Keyword</v>
-      </c>
-      <c r="G6" t="str">
-        <v>pushed to exit door</v>
-      </c>
-      <c r="H6" t="str">
-        <v>được đẩy ra cửa thoát</v>
-      </c>
-      <c r="I6" t="str">
-        <v>Ending</v>
-      </c>
       <c r="J6" t="str">
-        <v/>
+        <v>nặng</v>
       </c>
       <c r="K6" t="str">
         <v/>
@@ -720,10 +618,10 @@
         <v/>
       </c>
       <c r="N6" t="str">
-        <v/>
+        <v>Danh từ · Keyword</v>
       </c>
       <c r="O6" t="str">
-        <v/>
+        <v>Tính từ · Ending</v>
       </c>
       <c r="P6" t="str">
         <v/>
@@ -740,31 +638,31 @@
         <v>1</v>
       </c>
       <c r="B7">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C7">
         <v>2</v>
       </c>
       <c r="D7" t="str">
-        <v>flip-flops</v>
+        <v>customs officer</v>
       </c>
       <c r="E7" t="str">
-        <v>đôi dép lào</v>
+        <v>check</v>
       </c>
       <c r="F7" t="str">
-        <v>Keyword</v>
+        <v/>
       </c>
       <c r="G7" t="str">
-        <v>packed for the beach</v>
+        <v/>
       </c>
       <c r="H7" t="str">
-        <v>xếp sẵn cho chuyến đi biển</v>
+        <v/>
       </c>
       <c r="I7" t="str">
-        <v>Ending</v>
+        <v>nhân viên hải quan</v>
       </c>
       <c r="J7" t="str">
-        <v/>
+        <v>kiểm tra</v>
       </c>
       <c r="K7" t="str">
         <v/>
@@ -776,10 +674,10 @@
         <v/>
       </c>
       <c r="N7" t="str">
-        <v/>
+        <v>Danh từ · Keyword</v>
       </c>
       <c r="O7" t="str">
-        <v/>
+        <v>Động từ · Ending</v>
       </c>
       <c r="P7" t="str">
         <v/>
@@ -796,31 +694,31 @@
         <v>1</v>
       </c>
       <c r="B8">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C8">
         <v>2</v>
       </c>
       <c r="D8" t="str">
-        <v>check-in counter</v>
+        <v>sleeping bag</v>
       </c>
       <c r="E8" t="str">
-        <v>quầy làm thủ tục</v>
+        <v>warm</v>
       </c>
       <c r="F8" t="str">
-        <v>Keyword</v>
+        <v/>
       </c>
       <c r="G8" t="str">
-        <v>crowded with travelers</v>
+        <v/>
       </c>
       <c r="H8" t="str">
-        <v>chật kín khách du lịch</v>
+        <v/>
       </c>
       <c r="I8" t="str">
-        <v>Ending</v>
+        <v>túi ngủ</v>
       </c>
       <c r="J8" t="str">
-        <v/>
+        <v>ấm áp</v>
       </c>
       <c r="K8" t="str">
         <v/>
@@ -832,10 +730,10 @@
         <v/>
       </c>
       <c r="N8" t="str">
-        <v/>
+        <v>Danh từ · Keyword</v>
       </c>
       <c r="O8" t="str">
-        <v/>
+        <v>Tính từ · Ending</v>
       </c>
       <c r="P8" t="str">
         <v/>
@@ -852,31 +750,31 @@
         <v>1</v>
       </c>
       <c r="B9">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C9">
         <v>2</v>
       </c>
       <c r="D9" t="str">
-        <v>hotel address</v>
+        <v>hotel</v>
       </c>
       <c r="E9" t="str">
-        <v>địa chỉ khách sạn</v>
+        <v>book in advance</v>
       </c>
       <c r="F9" t="str">
-        <v>Keyword</v>
+        <v/>
       </c>
       <c r="G9" t="str">
-        <v>saved on phone</v>
+        <v/>
       </c>
       <c r="H9" t="str">
-        <v>được lưu trong điện thoại</v>
+        <v/>
       </c>
       <c r="I9" t="str">
-        <v>Ending</v>
+        <v>khách sạn</v>
       </c>
       <c r="J9" t="str">
-        <v/>
+        <v>đặt trước</v>
       </c>
       <c r="K9" t="str">
         <v/>
@@ -888,10 +786,10 @@
         <v/>
       </c>
       <c r="N9" t="str">
-        <v/>
+        <v>Danh từ · Keyword</v>
       </c>
       <c r="O9" t="str">
-        <v/>
+        <v>Động từ · Ending</v>
       </c>
       <c r="P9" t="str">
         <v/>
@@ -908,31 +806,31 @@
         <v>1</v>
       </c>
       <c r="B10">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C10">
         <v>2</v>
       </c>
       <c r="D10" t="str">
-        <v>painkillers</v>
+        <v>flight</v>
       </c>
       <c r="E10" t="str">
-        <v>thuốc giảm đau</v>
+        <v>delayed</v>
       </c>
       <c r="F10" t="str">
-        <v>Keyword</v>
+        <v/>
       </c>
       <c r="G10" t="str">
-        <v>taken after the flight</v>
+        <v/>
       </c>
       <c r="H10" t="str">
-        <v>được uống sau chuyến bay</v>
+        <v/>
       </c>
       <c r="I10" t="str">
-        <v>Ending</v>
+        <v>chuyến bay</v>
       </c>
       <c r="J10" t="str">
-        <v/>
+        <v>hoãn</v>
       </c>
       <c r="K10" t="str">
         <v/>
@@ -944,10 +842,10 @@
         <v/>
       </c>
       <c r="N10" t="str">
-        <v/>
+        <v>Danh từ · Keyword</v>
       </c>
       <c r="O10" t="str">
-        <v/>
+        <v>Tính từ · Ending</v>
       </c>
       <c r="P10" t="str">
         <v/>
@@ -964,31 +862,31 @@
         <v>1</v>
       </c>
       <c r="B11">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C11">
         <v>2</v>
       </c>
       <c r="D11" t="str">
-        <v>window seat</v>
+        <v>passport</v>
       </c>
       <c r="E11" t="str">
-        <v>ghế cạnh cửa sổ</v>
+        <v>forget</v>
       </c>
       <c r="F11" t="str">
-        <v>Keyword</v>
+        <v/>
       </c>
       <c r="G11" t="str">
-        <v>booked in advance</v>
+        <v/>
       </c>
       <c r="H11" t="str">
-        <v>đã được đặt chỗ trước</v>
+        <v/>
       </c>
       <c r="I11" t="str">
-        <v>Ending</v>
+        <v>hộ chiếu</v>
       </c>
       <c r="J11" t="str">
-        <v/>
+        <v>quên</v>
       </c>
       <c r="K11" t="str">
         <v/>
@@ -1000,10 +898,10 @@
         <v/>
       </c>
       <c r="N11" t="str">
-        <v/>
+        <v>Danh từ · Keyword</v>
       </c>
       <c r="O11" t="str">
-        <v/>
+        <v>Động từ · Ending</v>
       </c>
       <c r="P11" t="str">
         <v/>
@@ -1020,31 +918,31 @@
         <v>1</v>
       </c>
       <c r="B12">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C12">
         <v>2</v>
       </c>
       <c r="D12" t="str">
-        <v>departure time</v>
+        <v>suitcase</v>
       </c>
       <c r="E12" t="str">
-        <v>giờ máy bay cất cánh</v>
+        <v>lock</v>
       </c>
       <c r="F12" t="str">
-        <v>Keyword</v>
+        <v/>
       </c>
       <c r="G12" t="str">
-        <v>delayed by one hour</v>
+        <v/>
       </c>
       <c r="H12" t="str">
-        <v>bị hoãn lại một tiếng</v>
+        <v/>
       </c>
       <c r="I12" t="str">
-        <v>Ending</v>
+        <v>vali</v>
       </c>
       <c r="J12" t="str">
-        <v/>
+        <v>khóa</v>
       </c>
       <c r="K12" t="str">
         <v/>
@@ -1056,10 +954,10 @@
         <v/>
       </c>
       <c r="N12" t="str">
-        <v/>
+        <v>Danh từ · Keyword</v>
       </c>
       <c r="O12" t="str">
-        <v/>
+        <v>Động từ · Ending</v>
       </c>
       <c r="P12" t="str">
         <v/>
@@ -1076,31 +974,31 @@
         <v>1</v>
       </c>
       <c r="B13">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C13">
         <v>2</v>
       </c>
       <c r="D13" t="str">
-        <v>local night market</v>
+        <v>flip-flops</v>
       </c>
       <c r="E13" t="str">
-        <v>chợ đêm địa phương</v>
+        <v>beach trip</v>
       </c>
       <c r="F13" t="str">
-        <v>Keyword</v>
+        <v/>
       </c>
       <c r="G13" t="str">
-        <v>packed with food stalls</v>
+        <v/>
       </c>
       <c r="H13" t="str">
-        <v>đầy ắp các quầy ăn uống</v>
+        <v/>
       </c>
       <c r="I13" t="str">
-        <v>Ending</v>
+        <v>dép lào</v>
       </c>
       <c r="J13" t="str">
-        <v/>
+        <v>đi biển</v>
       </c>
       <c r="K13" t="str">
         <v/>
@@ -1112,10 +1010,10 @@
         <v/>
       </c>
       <c r="N13" t="str">
-        <v/>
+        <v>Danh từ · Keyword</v>
       </c>
       <c r="O13" t="str">
-        <v/>
+        <v>Danh từ · Ending</v>
       </c>
       <c r="P13" t="str">
         <v/>
@@ -1132,31 +1030,31 @@
         <v>1</v>
       </c>
       <c r="B14">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C14">
         <v>2</v>
       </c>
       <c r="D14" t="str">
-        <v>tuktuk ride</v>
+        <v>boarding gate</v>
       </c>
       <c r="E14" t="str">
-        <v>chuyến xe tuktuk</v>
+        <v>find</v>
       </c>
       <c r="F14" t="str">
-        <v>Keyword</v>
+        <v/>
       </c>
       <c r="G14" t="str">
-        <v>hailed near the station</v>
+        <v/>
       </c>
       <c r="H14" t="str">
-        <v>được vẫy gần ga tàu</v>
+        <v/>
       </c>
       <c r="I14" t="str">
-        <v>Ending</v>
+        <v>cửa khởi hành</v>
       </c>
       <c r="J14" t="str">
-        <v/>
+        <v>tìm</v>
       </c>
       <c r="K14" t="str">
         <v/>
@@ -1168,10 +1066,10 @@
         <v/>
       </c>
       <c r="N14" t="str">
-        <v/>
+        <v>Danh từ · Keyword</v>
       </c>
       <c r="O14" t="str">
-        <v/>
+        <v>Động từ · Ending</v>
       </c>
       <c r="P14" t="str">
         <v/>
@@ -1188,31 +1086,31 @@
         <v>1</v>
       </c>
       <c r="B15">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C15">
         <v>2</v>
       </c>
       <c r="D15" t="str">
-        <v>ancient temple</v>
+        <v>snacks</v>
       </c>
       <c r="E15" t="str">
-        <v>ngôi đền cổ kính</v>
+        <v>bring along</v>
       </c>
       <c r="F15" t="str">
-        <v>Keyword</v>
+        <v/>
       </c>
       <c r="G15" t="str">
-        <v>visited in early morning</v>
+        <v/>
       </c>
       <c r="H15" t="str">
-        <v>được ghé thăm từ sớm</v>
+        <v/>
       </c>
       <c r="I15" t="str">
-        <v>Ending</v>
+        <v>đồ ăn nhẹ</v>
       </c>
       <c r="J15" t="str">
-        <v/>
+        <v>mang theo</v>
       </c>
       <c r="K15" t="str">
         <v/>
@@ -1224,10 +1122,10 @@
         <v/>
       </c>
       <c r="N15" t="str">
-        <v/>
+        <v>Danh từ · Keyword</v>
       </c>
       <c r="O15" t="str">
-        <v/>
+        <v>Động từ · Ending</v>
       </c>
       <c r="P15" t="str">
         <v/>
@@ -1244,31 +1142,31 @@
         <v>1</v>
       </c>
       <c r="B16">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C16">
         <v>2</v>
       </c>
       <c r="D16" t="str">
-        <v>flight transit</v>
+        <v>layover time</v>
       </c>
       <c r="E16" t="str">
-        <v>chuyến bay quá cảnh</v>
+        <v>long</v>
       </c>
       <c r="F16" t="str">
-        <v>Keyword</v>
+        <v/>
       </c>
       <c r="G16" t="str">
-        <v>lasted four long hours</v>
+        <v/>
       </c>
       <c r="H16" t="str">
-        <v>kéo dài suốt bốn tiếng</v>
+        <v/>
       </c>
       <c r="I16" t="str">
-        <v>Ending</v>
+        <v>thời gian quá cảnh</v>
       </c>
       <c r="J16" t="str">
-        <v/>
+        <v>dài</v>
       </c>
       <c r="K16" t="str">
         <v/>
@@ -1280,10 +1178,10 @@
         <v/>
       </c>
       <c r="N16" t="str">
-        <v/>
+        <v>Danh từ · Keyword</v>
       </c>
       <c r="O16" t="str">
-        <v/>
+        <v>Tính từ · Ending</v>
       </c>
       <c r="P16" t="str">
         <v/>
@@ -1297,49 +1195,49 @@
     </row>
     <row r="17">
       <c r="A17">
+        <v>1</v>
+      </c>
+      <c r="B17">
+        <v>14</v>
+      </c>
+      <c r="C17">
         <v>2</v>
       </c>
-      <c r="B17">
-        <v>1</v>
-      </c>
-      <c r="C17">
-        <v>3</v>
-      </c>
       <c r="D17" t="str">
-        <v>rush hour detour</v>
+        <v>taxi driver</v>
       </c>
       <c r="E17" t="str">
-        <v>đường vòng giờ cao điểm</v>
+        <v>friendly</v>
       </c>
       <c r="F17" t="str">
-        <v>Keyword</v>
+        <v/>
       </c>
       <c r="G17" t="str">
-        <v>because of the</v>
+        <v/>
       </c>
       <c r="H17" t="str">
-        <v>chính vì...</v>
+        <v/>
       </c>
       <c r="I17" t="str">
-        <v>Logic word</v>
+        <v>tài xế taxi</v>
       </c>
       <c r="J17" t="str">
-        <v>missed final boarding</v>
+        <v>thân thiện</v>
       </c>
       <c r="K17" t="str">
-        <v>lỡ mất giờ lên máy bay</v>
+        <v/>
       </c>
       <c r="L17" t="str">
-        <v>Ending</v>
+        <v/>
       </c>
       <c r="M17" t="str">
         <v/>
       </c>
       <c r="N17" t="str">
-        <v/>
+        <v>Danh từ · Keyword</v>
       </c>
       <c r="O17" t="str">
-        <v/>
+        <v>Tính từ · Ending</v>
       </c>
       <c r="P17" t="str">
         <v/>
@@ -1353,49 +1251,49 @@
     </row>
     <row r="18">
       <c r="A18">
+        <v>1</v>
+      </c>
+      <c r="B18">
+        <v>15</v>
+      </c>
+      <c r="C18">
         <v>2</v>
       </c>
-      <c r="B18">
-        <v>2</v>
-      </c>
-      <c r="C18">
-        <v>3</v>
-      </c>
       <c r="D18" t="str">
-        <v>overslept in hotel</v>
+        <v>rice cooker</v>
       </c>
       <c r="E18" t="str">
-        <v>ngủ quên ở khách sạn</v>
+        <v>cook rice</v>
       </c>
       <c r="F18" t="str">
-        <v>Keyword</v>
+        <v/>
       </c>
       <c r="G18" t="str">
-        <v>as a result of</v>
+        <v/>
       </c>
       <c r="H18" t="str">
-        <v>kết quả là do...</v>
+        <v/>
       </c>
       <c r="I18" t="str">
-        <v>Logic word</v>
+        <v>nồi cơm điện</v>
       </c>
       <c r="J18" t="str">
-        <v>sprinted across terminal</v>
+        <v>nấu cơm</v>
       </c>
       <c r="K18" t="str">
-        <v>chạy thục mạng qua nhà ga</v>
+        <v/>
       </c>
       <c r="L18" t="str">
-        <v>Ending</v>
+        <v/>
       </c>
       <c r="M18" t="str">
         <v/>
       </c>
       <c r="N18" t="str">
-        <v/>
+        <v>Danh từ · Keyword</v>
       </c>
       <c r="O18" t="str">
-        <v/>
+        <v>Động từ · Ending</v>
       </c>
       <c r="P18" t="str">
         <v/>
@@ -1412,49 +1310,49 @@
         <v>2</v>
       </c>
       <c r="B19">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C19">
         <v>3</v>
       </c>
       <c r="D19" t="str">
-        <v>misread gate number</v>
+        <v>heavy luggage</v>
       </c>
       <c r="E19" t="str">
-        <v>đọc nhầm số cổng bay</v>
+        <v>therefore</v>
       </c>
       <c r="F19" t="str">
-        <v>Keyword</v>
+        <v>exhausted</v>
       </c>
       <c r="G19" t="str">
-        <v>and consequently</v>
+        <v/>
       </c>
       <c r="H19" t="str">
-        <v>và do đó đã...</v>
+        <v/>
       </c>
       <c r="I19" t="str">
-        <v>Logic word</v>
+        <v>hành lý nặng</v>
       </c>
       <c r="J19" t="str">
-        <v>waited at wrong gate</v>
+        <v>do đó</v>
       </c>
       <c r="K19" t="str">
-        <v>đứng chờ nhầm ở cổng khác</v>
+        <v>mệt lử</v>
       </c>
       <c r="L19" t="str">
-        <v>Ending</v>
+        <v/>
       </c>
       <c r="M19" t="str">
         <v/>
       </c>
       <c r="N19" t="str">
-        <v/>
+        <v>Danh từ · Keyword</v>
       </c>
       <c r="O19" t="str">
-        <v/>
+        <v>Từ nối · Logic word</v>
       </c>
       <c r="P19" t="str">
-        <v/>
+        <v>Tính từ · Ending</v>
       </c>
       <c r="Q19" t="str">
         <v/>
@@ -1468,49 +1366,49 @@
         <v>2</v>
       </c>
       <c r="B20">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C20">
         <v>3</v>
       </c>
       <c r="D20" t="str">
-        <v>terrible seasick feeling</v>
+        <v>passport renewal</v>
       </c>
       <c r="E20" t="str">
-        <v>cảm giác say sóng dữ dội</v>
+        <v>before that</v>
       </c>
       <c r="F20" t="str">
-        <v>Keyword</v>
+        <v>urgent</v>
       </c>
       <c r="G20" t="str">
-        <v>due to the</v>
+        <v/>
       </c>
       <c r="H20" t="str">
-        <v>bởi vì gặp phải...</v>
+        <v/>
       </c>
       <c r="I20" t="str">
-        <v>Logic word</v>
+        <v>gia hạn hộ chiếu</v>
       </c>
       <c r="J20" t="str">
-        <v>rested inside the cabin</v>
+        <v>trước đó</v>
       </c>
       <c r="K20" t="str">
-        <v>phải nằm nghỉ trong khoang tàu</v>
+        <v>khẩn cấp</v>
       </c>
       <c r="L20" t="str">
-        <v>Ending</v>
+        <v/>
       </c>
       <c r="M20" t="str">
         <v/>
       </c>
       <c r="N20" t="str">
-        <v/>
+        <v>Danh từ · Keyword</v>
       </c>
       <c r="O20" t="str">
-        <v/>
+        <v>Từ nối · Logic word</v>
       </c>
       <c r="P20" t="str">
-        <v/>
+        <v>Tính từ · Ending</v>
       </c>
       <c r="Q20" t="str">
         <v/>
@@ -1524,49 +1422,49 @@
         <v>2</v>
       </c>
       <c r="B21">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C21">
         <v>3</v>
       </c>
       <c r="D21" t="str">
-        <v>left luggage behind</v>
+        <v>flight delay</v>
       </c>
       <c r="E21" t="str">
-        <v>bỏ quên hành lý lại</v>
+        <v>meanwhile</v>
       </c>
       <c r="F21" t="str">
-        <v>Keyword</v>
+        <v>rest</v>
       </c>
       <c r="G21" t="str">
-        <v>right after realizing</v>
+        <v/>
       </c>
       <c r="H21" t="str">
-        <v>ngay sau khi nhận ra...</v>
+        <v/>
       </c>
       <c r="I21" t="str">
-        <v>Logic word</v>
+        <v>chuyến bay hoãn</v>
       </c>
       <c r="J21" t="str">
-        <v>ran back to customs</v>
+        <v>đồng thời</v>
       </c>
       <c r="K21" t="str">
-        <v>chạy vội quay lại hải quan</v>
+        <v>nghỉ ngơi</v>
       </c>
       <c r="L21" t="str">
-        <v>Ending</v>
+        <v/>
       </c>
       <c r="M21" t="str">
         <v/>
       </c>
       <c r="N21" t="str">
-        <v/>
+        <v>Danh từ · Keyword</v>
       </c>
       <c r="O21" t="str">
-        <v/>
+        <v>Từ nối · Logic word</v>
       </c>
       <c r="P21" t="str">
-        <v/>
+        <v>Động từ · Ending</v>
       </c>
       <c r="Q21" t="str">
         <v/>
@@ -1580,49 +1478,49 @@
         <v>2</v>
       </c>
       <c r="B22">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C22">
         <v>3</v>
       </c>
       <c r="D22" t="str">
-        <v>severe food allergy</v>
+        <v>taxi fare</v>
       </c>
       <c r="E22" t="str">
-        <v>dị ứng thức ăn nghiêm trọng</v>
+        <v>in addition</v>
       </c>
       <c r="F22" t="str">
-        <v>Keyword</v>
+        <v>expensive</v>
       </c>
       <c r="G22" t="str">
-        <v>owing to</v>
+        <v/>
       </c>
       <c r="H22" t="str">
-        <v>bởi vì dính phải...</v>
+        <v/>
       </c>
       <c r="I22" t="str">
-        <v>Logic word</v>
+        <v>tiền taxi</v>
       </c>
       <c r="J22" t="str">
-        <v>checked local hospital</v>
+        <v>hơn nữa</v>
       </c>
       <c r="K22" t="str">
-        <v>phải vào viện địa phương kiểm tra</v>
+        <v>đắt đỏ</v>
       </c>
       <c r="L22" t="str">
-        <v>Ending</v>
+        <v/>
       </c>
       <c r="M22" t="str">
         <v/>
       </c>
       <c r="N22" t="str">
-        <v/>
+        <v>Danh từ · Keyword</v>
       </c>
       <c r="O22" t="str">
-        <v/>
+        <v>Từ nối · Logic word</v>
       </c>
       <c r="P22" t="str">
-        <v/>
+        <v>Tính từ · Ending</v>
       </c>
       <c r="Q22" t="str">
         <v/>
@@ -1636,49 +1534,49 @@
         <v>2</v>
       </c>
       <c r="B23">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C23">
         <v>3</v>
       </c>
       <c r="D23" t="str">
-        <v>lost hotel address</v>
+        <v>boarding gate</v>
       </c>
       <c r="E23" t="str">
-        <v>làm mất địa chỉ khách sạn</v>
+        <v>next</v>
       </c>
       <c r="F23" t="str">
-        <v>Keyword</v>
+        <v>sprint</v>
       </c>
       <c r="G23" t="str">
-        <v>so in order to</v>
+        <v/>
       </c>
       <c r="H23" t="str">
-        <v>nên để có thể...</v>
+        <v/>
       </c>
       <c r="I23" t="str">
-        <v>Logic word</v>
+        <v>cửa ra máy bay</v>
       </c>
       <c r="J23" t="str">
-        <v>asked nearby locals</v>
+        <v>tiếp theo</v>
       </c>
       <c r="K23" t="str">
-        <v>hỏi thăm người dân xung quanh</v>
+        <v>chạy nước rút</v>
       </c>
       <c r="L23" t="str">
-        <v>Ending</v>
+        <v/>
       </c>
       <c r="M23" t="str">
         <v/>
       </c>
       <c r="N23" t="str">
-        <v/>
+        <v>Danh từ · Keyword</v>
       </c>
       <c r="O23" t="str">
-        <v/>
+        <v>Từ nối · Logic word</v>
       </c>
       <c r="P23" t="str">
-        <v/>
+        <v>Động từ · Ending</v>
       </c>
       <c r="Q23" t="str">
         <v/>
@@ -1692,49 +1590,49 @@
         <v>2</v>
       </c>
       <c r="B24">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C24">
         <v>3</v>
       </c>
       <c r="D24" t="str">
-        <v>airport power outage</v>
+        <v>window seat</v>
       </c>
       <c r="E24" t="str">
-        <v>sự cố mất điện sân bay</v>
+        <v>otherwise</v>
       </c>
       <c r="F24" t="str">
-        <v>Keyword</v>
+        <v>cramped</v>
       </c>
       <c r="G24" t="str">
-        <v>which suddenly led to</v>
+        <v/>
       </c>
       <c r="H24" t="str">
-        <v>điều đó bất ngờ dẫn đến...</v>
+        <v/>
       </c>
       <c r="I24" t="str">
-        <v>Logic word</v>
+        <v>ghế cạnh cửa sổ</v>
       </c>
       <c r="J24" t="str">
-        <v>halted luggage screening</v>
+        <v>nếu không</v>
       </c>
       <c r="K24" t="str">
-        <v>đình trệ khâu soi chiếu hành lý</v>
+        <v>chật chội</v>
       </c>
       <c r="L24" t="str">
-        <v>Ending</v>
+        <v/>
       </c>
       <c r="M24" t="str">
         <v/>
       </c>
       <c r="N24" t="str">
-        <v/>
+        <v>Danh từ · Keyword</v>
       </c>
       <c r="O24" t="str">
-        <v/>
+        <v>Từ nối · Logic word</v>
       </c>
       <c r="P24" t="str">
-        <v/>
+        <v>Tính từ · Ending</v>
       </c>
       <c r="Q24" t="str">
         <v/>
@@ -1748,49 +1646,49 @@
         <v>2</v>
       </c>
       <c r="B25">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C25">
         <v>3</v>
       </c>
       <c r="D25" t="str">
-        <v>dead phone battery</v>
+        <v>travel insurance</v>
       </c>
       <c r="E25" t="str">
-        <v>điện thoại cạn sạch pin</v>
+        <v>if</v>
       </c>
       <c r="F25" t="str">
-        <v>Keyword</v>
+        <v>secure</v>
       </c>
       <c r="G25" t="str">
-        <v>since I had</v>
+        <v/>
       </c>
       <c r="H25" t="str">
-        <v>vì bản thân bị...</v>
+        <v/>
       </c>
       <c r="I25" t="str">
-        <v>Logic word</v>
+        <v>bảo hiểm du lịch</v>
       </c>
       <c r="J25" t="str">
-        <v>searched for charging station</v>
+        <v>nếu</v>
       </c>
       <c r="K25" t="str">
-        <v>ráo riết tìm trạm sạc điện thoại</v>
+        <v>an tâm</v>
       </c>
       <c r="L25" t="str">
-        <v>Ending</v>
+        <v/>
       </c>
       <c r="M25" t="str">
         <v/>
       </c>
       <c r="N25" t="str">
-        <v/>
+        <v>Danh từ · Keyword</v>
       </c>
       <c r="O25" t="str">
-        <v/>
+        <v>Từ nối · Logic word</v>
       </c>
       <c r="P25" t="str">
-        <v/>
+        <v>Tính từ · Ending</v>
       </c>
       <c r="Q25" t="str">
         <v/>
@@ -1804,49 +1702,49 @@
         <v>2</v>
       </c>
       <c r="B26">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C26">
         <v>3</v>
       </c>
       <c r="D26" t="str">
-        <v>broken suitcase wheel</v>
+        <v>broken wheel</v>
       </c>
       <c r="E26" t="str">
-        <v>bánh xe vali bị gãy</v>
+        <v>nevertheless</v>
       </c>
       <c r="F26" t="str">
-        <v>Keyword</v>
+        <v>manageable</v>
       </c>
       <c r="G26" t="str">
-        <v>despite having a</v>
+        <v/>
       </c>
       <c r="H26" t="str">
-        <v>mặc dù bị...</v>
+        <v/>
       </c>
       <c r="I26" t="str">
-        <v>Logic word</v>
+        <v>bánh xe bị gãy</v>
       </c>
       <c r="J26" t="str">
-        <v>dragged it through lobby</v>
+        <v>dù vậy</v>
       </c>
       <c r="K26" t="str">
-        <v>vẫn kéo lê qua sảnh lớn</v>
+        <v>xoay xở được</v>
       </c>
       <c r="L26" t="str">
-        <v>Ending</v>
+        <v/>
       </c>
       <c r="M26" t="str">
         <v/>
       </c>
       <c r="N26" t="str">
-        <v/>
+        <v>Danh từ · Keyword</v>
       </c>
       <c r="O26" t="str">
-        <v/>
+        <v>Từ nối · Logic word</v>
       </c>
       <c r="P26" t="str">
-        <v/>
+        <v>Tính từ · Ending</v>
       </c>
       <c r="Q26" t="str">
         <v/>
@@ -1860,49 +1758,49 @@
         <v>2</v>
       </c>
       <c r="B27">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C27">
         <v>3</v>
       </c>
       <c r="D27" t="str">
-        <v>unexpected flight cancellation</v>
+        <v>foreign currency</v>
       </c>
       <c r="E27" t="str">
-        <v>chuyến bay bị hủy bất ngờ</v>
+        <v>in other words</v>
       </c>
       <c r="F27" t="str">
-        <v>Keyword</v>
+        <v>exchange</v>
       </c>
       <c r="G27" t="str">
-        <v>prompted by</v>
+        <v/>
       </c>
       <c r="H27" t="str">
-        <v>bắt nguồn từ việc...</v>
+        <v/>
       </c>
       <c r="I27" t="str">
-        <v>Logic word</v>
+        <v>ngoại tệ</v>
       </c>
       <c r="J27" t="str">
-        <v>queued for rebooking</v>
+        <v>nói cách khác</v>
       </c>
       <c r="K27" t="str">
-        <v>xếp hàng đổi vé máy bay</v>
+        <v>đổi tiền</v>
       </c>
       <c r="L27" t="str">
-        <v>Ending</v>
+        <v/>
       </c>
       <c r="M27" t="str">
         <v/>
       </c>
       <c r="N27" t="str">
-        <v/>
+        <v>Danh từ · Keyword</v>
       </c>
       <c r="O27" t="str">
-        <v/>
+        <v>Từ nối · Logic word</v>
       </c>
       <c r="P27" t="str">
-        <v/>
+        <v>Động từ · Ending</v>
       </c>
       <c r="Q27" t="str">
         <v/>
@@ -1916,49 +1814,49 @@
         <v>2</v>
       </c>
       <c r="B28">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C28">
         <v>3</v>
       </c>
       <c r="D28" t="str">
-        <v>confusing airport signs</v>
+        <v>hotel room</v>
       </c>
       <c r="E28" t="str">
-        <v>biển chỉ dẫn khó hiểu</v>
+        <v>eventually</v>
       </c>
       <c r="F28" t="str">
-        <v>Keyword</v>
+        <v>confirmed</v>
       </c>
       <c r="G28" t="str">
-        <v>because of those</v>
+        <v/>
       </c>
       <c r="H28" t="str">
-        <v>vì những tấm biển đó...</v>
+        <v/>
       </c>
       <c r="I28" t="str">
-        <v>Logic word</v>
+        <v>phòng khách sạn</v>
       </c>
       <c r="J28" t="str">
-        <v>took long detour</v>
+        <v>sau cùng</v>
       </c>
       <c r="K28" t="str">
-        <v>đi một vòng đường thật xa</v>
+        <v>xác nhận</v>
       </c>
       <c r="L28" t="str">
-        <v>Ending</v>
+        <v/>
       </c>
       <c r="M28" t="str">
         <v/>
       </c>
       <c r="N28" t="str">
-        <v/>
+        <v>Danh từ · Keyword</v>
       </c>
       <c r="O28" t="str">
-        <v/>
+        <v>Từ nối · Logic word</v>
       </c>
       <c r="P28" t="str">
-        <v/>
+        <v>Tính từ · Ending</v>
       </c>
       <c r="Q28" t="str">
         <v/>
@@ -1972,49 +1870,49 @@
         <v>2</v>
       </c>
       <c r="B29">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C29">
         <v>3</v>
       </c>
       <c r="D29" t="str">
-        <v>overweight baggage fee</v>
+        <v>street market</v>
       </c>
       <c r="E29" t="str">
-        <v>phí phạt hành lý quá ký</v>
+        <v>however</v>
       </c>
       <c r="F29" t="str">
-        <v>Keyword</v>
+        <v>crowded</v>
       </c>
       <c r="G29" t="str">
-        <v>in order to avoid</v>
+        <v/>
       </c>
       <c r="H29" t="str">
-        <v>để tránh bị...</v>
+        <v/>
       </c>
       <c r="I29" t="str">
-        <v>Logic word</v>
+        <v>chợ đường phố</v>
       </c>
       <c r="J29" t="str">
-        <v>rearranged winter coats</v>
+        <v>tuy nhiên</v>
       </c>
       <c r="K29" t="str">
-        <v>phải mở ra soạn lại áo ấm</v>
+        <v>đông đúc</v>
       </c>
       <c r="L29" t="str">
-        <v>Ending</v>
+        <v/>
       </c>
       <c r="M29" t="str">
         <v/>
       </c>
       <c r="N29" t="str">
-        <v/>
+        <v>Danh từ · Keyword</v>
       </c>
       <c r="O29" t="str">
-        <v/>
+        <v>Từ nối · Logic word</v>
       </c>
       <c r="P29" t="str">
-        <v/>
+        <v>Tính từ · Ending</v>
       </c>
       <c r="Q29" t="str">
         <v/>
@@ -2028,49 +1926,49 @@
         <v>2</v>
       </c>
       <c r="B30">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C30">
         <v>3</v>
       </c>
       <c r="D30" t="str">
-        <v>spilled hot coffee</v>
+        <v>transit flight</v>
       </c>
       <c r="E30" t="str">
-        <v>lỡ làm đổ cà phê nóng</v>
+        <v>as long as</v>
       </c>
       <c r="F30" t="str">
-        <v>Keyword</v>
+        <v>on time</v>
       </c>
       <c r="G30" t="str">
-        <v>right before the</v>
+        <v/>
       </c>
       <c r="H30" t="str">
-        <v>ngay trước khi...</v>
+        <v/>
       </c>
       <c r="I30" t="str">
-        <v>Logic word</v>
+        <v>chuyến bay quá cảnh</v>
       </c>
       <c r="J30" t="str">
-        <v>changed into clean shirt</v>
+        <v>miễn là</v>
       </c>
       <c r="K30" t="str">
-        <v>phải thay ngay áo sạch mới</v>
+        <v>đúng giờ</v>
       </c>
       <c r="L30" t="str">
-        <v>Ending</v>
+        <v/>
       </c>
       <c r="M30" t="str">
         <v/>
       </c>
       <c r="N30" t="str">
-        <v/>
+        <v>Danh từ · Keyword</v>
       </c>
       <c r="O30" t="str">
-        <v/>
+        <v>Từ nối · Logic word</v>
       </c>
       <c r="P30" t="str">
-        <v/>
+        <v>Tính từ · Ending</v>
       </c>
       <c r="Q30" t="str">
         <v/>
@@ -2084,49 +1982,49 @@
         <v>2</v>
       </c>
       <c r="B31">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C31">
         <v>3</v>
       </c>
       <c r="D31" t="str">
-        <v>lost boarding pass</v>
+        <v>power bank</v>
       </c>
       <c r="E31" t="str">
-        <v>làm rơi thẻ lên tàu bay</v>
+        <v>for example</v>
       </c>
       <c r="F31" t="str">
-        <v>Keyword</v>
+        <v>essential</v>
       </c>
       <c r="G31" t="str">
-        <v>therefore we had to</v>
+        <v/>
       </c>
       <c r="H31" t="str">
-        <v>vì thế chúng tôi đành phải...</v>
+        <v/>
       </c>
       <c r="I31" t="str">
-        <v>Logic word</v>
+        <v>sạc dự phòng</v>
       </c>
       <c r="J31" t="str">
-        <v>request emergency reprint</v>
+        <v>ví dụ</v>
       </c>
       <c r="K31" t="str">
-        <v>xin in lại vé khẩn cấp</v>
+        <v>thiết yếu</v>
       </c>
       <c r="L31" t="str">
-        <v>Ending</v>
+        <v/>
       </c>
       <c r="M31" t="str">
         <v/>
       </c>
       <c r="N31" t="str">
-        <v/>
+        <v>Danh từ · Keyword</v>
       </c>
       <c r="O31" t="str">
-        <v/>
+        <v>Từ nối · Logic word</v>
       </c>
       <c r="P31" t="str">
-        <v/>
+        <v>Tính từ · Ending</v>
       </c>
       <c r="Q31" t="str">
         <v/>
@@ -2137,52 +2035,52 @@
     </row>
     <row r="32">
       <c r="A32">
+        <v>2</v>
+      </c>
+      <c r="B32">
+        <v>14</v>
+      </c>
+      <c r="C32">
         <v>3</v>
       </c>
-      <c r="B32">
-        <v>1</v>
-      </c>
-      <c r="C32">
-        <v>4</v>
-      </c>
       <c r="D32" t="str">
-        <v>customs checkpoint</v>
+        <v>sudden rain</v>
       </c>
       <c r="E32" t="str">
-        <v>khu vực kiểm tra hải quan</v>
+        <v>then</v>
       </c>
       <c r="F32" t="str">
-        <v>Keyword</v>
+        <v>take shelter</v>
       </c>
       <c r="G32" t="str">
-        <v>approaching the</v>
+        <v/>
       </c>
       <c r="H32" t="str">
-        <v>khi tiến vào...</v>
+        <v/>
       </c>
       <c r="I32" t="str">
-        <v>Logic word</v>
+        <v>mưa bất chợt</v>
       </c>
       <c r="J32" t="str">
-        <v>stern-looking officer</v>
+        <v>sau đó</v>
       </c>
       <c r="K32" t="str">
-        <v>viên chức mặt mày nghiêm nghị</v>
+        <v>trú mưa</v>
       </c>
       <c r="L32" t="str">
-        <v>Fancy word</v>
+        <v/>
       </c>
       <c r="M32" t="str">
-        <v>scrutinized every single stamp</v>
+        <v/>
       </c>
       <c r="N32" t="str">
-        <v>săm soi kiểm tra từng con dấu</v>
+        <v>Danh từ · Keyword</v>
       </c>
       <c r="O32" t="str">
-        <v>Ending</v>
+        <v>Từ nối · Logic word</v>
       </c>
       <c r="P32" t="str">
-        <v/>
+        <v>Động từ · Ending</v>
       </c>
       <c r="Q32" t="str">
         <v/>
@@ -2193,52 +2091,52 @@
     </row>
     <row r="33">
       <c r="A33">
+        <v>2</v>
+      </c>
+      <c r="B33">
+        <v>15</v>
+      </c>
+      <c r="C33">
         <v>3</v>
       </c>
-      <c r="B33">
-        <v>2</v>
-      </c>
-      <c r="C33">
-        <v>4</v>
-      </c>
       <c r="D33" t="str">
-        <v>trolley jam</v>
+        <v>tour guide</v>
       </c>
       <c r="E33" t="str">
-        <v>ùn tắc xe đẩy hàng</v>
+        <v>besides</v>
       </c>
       <c r="F33" t="str">
-        <v>Keyword</v>
+        <v>knowledgeable</v>
       </c>
       <c r="G33" t="str">
-        <v>amid the</v>
+        <v/>
       </c>
       <c r="H33" t="str">
-        <v>ngay giữa...</v>
+        <v/>
       </c>
       <c r="I33" t="str">
-        <v>Logic word</v>
+        <v>hướng dẫn viên</v>
       </c>
       <c r="J33" t="str">
-        <v>chaotic baggage claim</v>
+        <v>ngoài ra</v>
       </c>
       <c r="K33" t="str">
-        <v>khu trả hành lý hỗn loạn</v>
+        <v>am hiểu</v>
       </c>
       <c r="L33" t="str">
-        <v>Fancy word</v>
+        <v/>
       </c>
       <c r="M33" t="str">
-        <v>retrieved heavy backpack</v>
+        <v/>
       </c>
       <c r="N33" t="str">
-        <v>kéo được chiếc balo nặng ra</v>
+        <v>Danh từ · Keyword</v>
       </c>
       <c r="O33" t="str">
-        <v>Ending</v>
+        <v>Từ nối · Logic word</v>
       </c>
       <c r="P33" t="str">
-        <v/>
+        <v>Tính từ · Ending</v>
       </c>
       <c r="Q33" t="str">
         <v/>
@@ -2252,52 +2150,52 @@
         <v>3</v>
       </c>
       <c r="B34">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C34">
         <v>4</v>
       </c>
       <c r="D34" t="str">
-        <v>overseas detour</v>
+        <v>customs check</v>
       </c>
       <c r="E34" t="str">
-        <v>chuyến đi đường vòng nơi xứ người</v>
+        <v>while</v>
       </c>
       <c r="F34" t="str">
-        <v>Keyword</v>
+        <v>red flag</v>
       </c>
       <c r="G34" t="str">
-        <v>following an</v>
+        <v>strict</v>
       </c>
       <c r="H34" t="str">
-        <v>sau khi theo một...</v>
+        <v/>
       </c>
       <c r="I34" t="str">
-        <v>Logic word</v>
+        <v>kiểm tra hải quan</v>
       </c>
       <c r="J34" t="str">
-        <v>unfamiliar country alley</v>
+        <v>trong khi</v>
       </c>
       <c r="K34" t="str">
-        <v>con hẻm lạ hoắc miền quê</v>
+        <v>dấu hiệu khả nghi</v>
       </c>
       <c r="L34" t="str">
-        <v>Fancy word</v>
+        <v>nghiêm ngặt</v>
       </c>
       <c r="M34" t="str">
-        <v>stumbled upon night market</v>
+        <v/>
       </c>
       <c r="N34" t="str">
-        <v>tình cờ lạc vào khu chợ đêm</v>
+        <v>Danh từ · Keyword</v>
       </c>
       <c r="O34" t="str">
-        <v>Ending</v>
+        <v>Từ nối · Logic word</v>
       </c>
       <c r="P34" t="str">
-        <v/>
+        <v>Ẩn dụ · Fancy word</v>
       </c>
       <c r="Q34" t="str">
-        <v/>
+        <v>Tính từ · Ending</v>
       </c>
       <c r="R34" t="str">
         <v/>
@@ -2308,52 +2206,52 @@
         <v>3</v>
       </c>
       <c r="B35">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C35">
         <v>4</v>
       </c>
       <c r="D35" t="str">
-        <v>severe carsickness</v>
+        <v>airport terminal</v>
       </c>
       <c r="E35" t="str">
-        <v>cơn say xe dữ dội</v>
+        <v>however</v>
       </c>
       <c r="F35" t="str">
-        <v>Keyword</v>
+        <v>lifeline</v>
       </c>
       <c r="G35" t="str">
-        <v>suffering from</v>
+        <v>helpful</v>
       </c>
       <c r="H35" t="str">
-        <v>bị hành hạ bởi...</v>
+        <v/>
       </c>
       <c r="I35" t="str">
-        <v>Logic word</v>
+        <v>nhà ga sân bay</v>
       </c>
       <c r="J35" t="str">
-        <v>winding mountain pass</v>
+        <v>tuy nhiên</v>
       </c>
       <c r="K35" t="str">
-        <v>đoạn đèo quanh co uốn khúc</v>
+        <v>phao cứu trợ</v>
       </c>
       <c r="L35" t="str">
-        <v>Fancy word</v>
+        <v>hữu ích</v>
       </c>
       <c r="M35" t="str">
-        <v>swallowed two painkillers</v>
+        <v/>
       </c>
       <c r="N35" t="str">
-        <v>uống liền hai viên thuốc giảm đau</v>
+        <v>Danh từ · Keyword</v>
       </c>
       <c r="O35" t="str">
-        <v>Ending</v>
+        <v>Từ nối · Logic word</v>
       </c>
       <c r="P35" t="str">
-        <v/>
+        <v>Ẩn dụ · Fancy word</v>
       </c>
       <c r="Q35" t="str">
-        <v/>
+        <v>Tính từ · Ending</v>
       </c>
       <c r="R35" t="str">
         <v/>
@@ -2364,52 +2262,52 @@
         <v>3</v>
       </c>
       <c r="B36">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C36">
         <v>4</v>
       </c>
       <c r="D36" t="str">
-        <v>delayed departure</v>
+        <v>Which flight</v>
       </c>
       <c r="E36" t="str">
-        <v>giờ cất cánh bị trễ</v>
+        <v>otherwise</v>
       </c>
       <c r="F36" t="str">
-        <v>Keyword</v>
+        <v>last call</v>
       </c>
       <c r="G36" t="str">
-        <v>irritated by the</v>
+        <v>missed</v>
       </c>
       <c r="H36" t="str">
-        <v>bực mình vì...</v>
+        <v/>
       </c>
       <c r="I36" t="str">
-        <v>Logic word</v>
+        <v>Chuyến bay nào</v>
       </c>
       <c r="J36" t="str">
-        <v>prolonged technical glitch</v>
+        <v>nếu không</v>
       </c>
       <c r="K36" t="str">
-        <v>sự cố kỹ thuật kéo dài lê thê</v>
+        <v>loa gọi chót</v>
       </c>
       <c r="L36" t="str">
-        <v>Fancy word</v>
+        <v>bị lỡ</v>
       </c>
       <c r="M36" t="str">
-        <v>dozed in sleeping bag</v>
+        <v/>
       </c>
       <c r="N36" t="str">
-        <v>chợp mắt luôn trong túi ngủ</v>
+        <v>Cụm nghi vấn · WH word</v>
       </c>
       <c r="O36" t="str">
-        <v>Ending</v>
+        <v>Từ nối · Logic word</v>
       </c>
       <c r="P36" t="str">
-        <v/>
+        <v>Cụm gợi hình · Fancy word</v>
       </c>
       <c r="Q36" t="str">
-        <v/>
+        <v>Tính từ · Ending</v>
       </c>
       <c r="R36" t="str">
         <v/>
@@ -2420,52 +2318,52 @@
         <v>3</v>
       </c>
       <c r="B37">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C37">
         <v>4</v>
       </c>
       <c r="D37" t="str">
-        <v>lost room key</v>
+        <v>lost baggage</v>
       </c>
       <c r="E37" t="str">
-        <v>chìa khóa phòng biến mất</v>
+        <v>therefore</v>
       </c>
       <c r="F37" t="str">
-        <v>Keyword</v>
+        <v>headache</v>
       </c>
       <c r="G37" t="str">
-        <v>frantically realizing</v>
+        <v>stressful</v>
       </c>
       <c r="H37" t="str">
-        <v>hốt hoảng phát hiện...</v>
+        <v/>
       </c>
       <c r="I37" t="str">
-        <v>Logic word</v>
+        <v>thất lạc hành lý</v>
       </c>
       <c r="J37" t="str">
-        <v>unlocked hotel suite</v>
+        <v>do đó</v>
       </c>
       <c r="K37" t="str">
-        <v>căn phòng khách sạn chưa khóa</v>
+        <v>cơn đau đầu</v>
       </c>
       <c r="L37" t="str">
-        <v>Fancy word</v>
+        <v>căng thẳng</v>
       </c>
       <c r="M37" t="str">
-        <v>alerted front desk manager</v>
+        <v/>
       </c>
       <c r="N37" t="str">
-        <v>báo ngay cho quản lý lễ tân</v>
+        <v>Danh từ · Keyword</v>
       </c>
       <c r="O37" t="str">
-        <v>Ending</v>
+        <v>Từ nối · Logic word</v>
       </c>
       <c r="P37" t="str">
-        <v/>
+        <v>Ẩn dụ · Fancy word</v>
       </c>
       <c r="Q37" t="str">
-        <v/>
+        <v>Tính từ · Ending</v>
       </c>
       <c r="R37" t="str">
         <v/>
@@ -2476,52 +2374,52 @@
         <v>3</v>
       </c>
       <c r="B38">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C38">
         <v>4</v>
       </c>
       <c r="D38" t="str">
-        <v>aisle seat swap</v>
+        <v>flight cancellation</v>
       </c>
       <c r="E38" t="str">
-        <v>đổi chỗ ngồi gần lối đi</v>
+        <v>in contrast</v>
       </c>
       <c r="F38" t="str">
-        <v>Keyword</v>
+        <v>dead stop</v>
       </c>
       <c r="G38" t="str">
-        <v>politely requesting an</v>
+        <v>refunded</v>
       </c>
       <c r="H38" t="str">
-        <v>lịch sự mở lời xin...</v>
+        <v/>
       </c>
       <c r="I38" t="str">
-        <v>Logic word</v>
+        <v>chuyến bay bị hủy</v>
       </c>
       <c r="J38" t="str">
-        <v>accommodating flight attendant</v>
+        <v>ngược lại</v>
       </c>
       <c r="K38" t="str">
-        <v>tiếp viên hàng không niềm nở</v>
+        <v>dừng hẳn</v>
       </c>
       <c r="L38" t="str">
-        <v>Fancy word</v>
+        <v>được bồi hoàn</v>
       </c>
       <c r="M38" t="str">
-        <v>stretched tired legs comfortably</v>
+        <v/>
       </c>
       <c r="N38" t="str">
-        <v>duỗi thẳng chân thoải mái nghỉ ngơi</v>
+        <v>Danh từ · Keyword</v>
       </c>
       <c r="O38" t="str">
-        <v>Ending</v>
+        <v>Từ nối · Logic word</v>
       </c>
       <c r="P38" t="str">
-        <v/>
+        <v>Ẩn dụ · Fancy word</v>
       </c>
       <c r="Q38" t="str">
-        <v/>
+        <v>Tính từ · Ending</v>
       </c>
       <c r="R38" t="str">
         <v/>
@@ -2532,52 +2430,52 @@
         <v>3</v>
       </c>
       <c r="B39">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C39">
         <v>4</v>
       </c>
       <c r="D39" t="str">
-        <v>misplaced passport</v>
+        <v>Why delay</v>
       </c>
       <c r="E39" t="str">
-        <v>để thất lạc cuốn hộ chiếu</v>
+        <v>finally</v>
       </c>
       <c r="F39" t="str">
-        <v>Keyword</v>
+        <v>safe harbor</v>
       </c>
       <c r="G39" t="str">
-        <v>panicking over</v>
+        <v>relieved</v>
       </c>
       <c r="H39" t="str">
-        <v>hoảng loạn vì...</v>
+        <v/>
       </c>
       <c r="I39" t="str">
-        <v>Logic word</v>
+        <v>Tại sao lại hoãn</v>
       </c>
       <c r="J39" t="str">
-        <v>essential travel credential</v>
+        <v>sau cùng</v>
       </c>
       <c r="K39" t="str">
-        <v>giấy tờ xuất ngoại quan trọng nhất</v>
+        <v>bến đỗ an toàn</v>
       </c>
       <c r="L39" t="str">
-        <v>Fancy word</v>
+        <v>thở phào</v>
       </c>
       <c r="M39" t="str">
-        <v>checked back pocket thoroughly</v>
+        <v/>
       </c>
       <c r="N39" t="str">
-        <v>lục tung kỹ lại túi quần sau</v>
+        <v>Cụm nghi vấn · WH word</v>
       </c>
       <c r="O39" t="str">
-        <v>Ending</v>
+        <v>Từ nối · Logic word</v>
       </c>
       <c r="P39" t="str">
-        <v/>
+        <v>Ẩn dụ · Fancy word</v>
       </c>
       <c r="Q39" t="str">
-        <v/>
+        <v>Tính từ · Ending</v>
       </c>
       <c r="R39" t="str">
         <v/>
@@ -2588,52 +2486,52 @@
         <v>3</v>
       </c>
       <c r="B40">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C40">
         <v>4</v>
       </c>
       <c r="D40" t="str">
-        <v>tuktuk scam</v>
+        <v>overseas travel</v>
       </c>
       <c r="E40" t="str">
-        <v>cú lừa cước xe tuktuk</v>
+        <v>as long as</v>
       </c>
       <c r="F40" t="str">
-        <v>Keyword</v>
+        <v>Better safe than sorry</v>
       </c>
       <c r="G40" t="str">
-        <v>wary of a</v>
+        <v>prepared</v>
       </c>
       <c r="H40" t="str">
-        <v>cảnh giác trước...</v>
+        <v/>
       </c>
       <c r="I40" t="str">
-        <v>Logic word</v>
+        <v>du lịch nước ngoài</v>
       </c>
       <c r="J40" t="str">
-        <v>suspiciously steep price</v>
+        <v>miễn là</v>
       </c>
       <c r="K40" t="str">
-        <v>mức giá cao một cách đáng ngờ</v>
+        <v>cẩn tắc vô áy náy</v>
       </c>
       <c r="L40" t="str">
-        <v>Fancy word</v>
+        <v>chuẩn bị kỹ</v>
       </c>
       <c r="M40" t="str">
-        <v>firmly bargained fare down</v>
+        <v/>
       </c>
       <c r="N40" t="str">
-        <v>nhất quyết trả giá xuống đúng mức</v>
+        <v>Danh từ · Keyword</v>
       </c>
       <c r="O40" t="str">
-        <v>Ending</v>
+        <v>Từ nối · Logic word</v>
       </c>
       <c r="P40" t="str">
-        <v/>
+        <v>Tục ngữ · Proverb</v>
       </c>
       <c r="Q40" t="str">
-        <v/>
+        <v>Tính từ · Ending</v>
       </c>
       <c r="R40" t="str">
         <v/>
@@ -2644,52 +2542,52 @@
         <v>3</v>
       </c>
       <c r="B41">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C41">
         <v>4</v>
       </c>
       <c r="D41" t="str">
-        <v>monsoon downpour</v>
+        <v>midnight layover</v>
       </c>
       <c r="E41" t="str">
-        <v>trận mưa rào nhiệt đới tầm tã</v>
+        <v>meanwhile</v>
       </c>
       <c r="F41" t="str">
-        <v>Keyword</v>
+        <v>empty chairs</v>
       </c>
       <c r="G41" t="str">
-        <v>trapped under the</v>
+        <v>freezing</v>
       </c>
       <c r="H41" t="str">
-        <v>mắc kẹt dưới...</v>
+        <v/>
       </c>
       <c r="I41" t="str">
-        <v>Logic word</v>
+        <v>quá cảnh nửa đêm</v>
       </c>
       <c r="J41" t="str">
-        <v>crumbling ancient pagoda</v>
+        <v>đồng thời</v>
       </c>
       <c r="K41" t="str">
-        <v>mái chùa cổ kính rêu phong</v>
+        <v>ghế trống trơn</v>
       </c>
       <c r="L41" t="str">
-        <v>Fancy word</v>
+        <v>lạnh cóng</v>
       </c>
       <c r="M41" t="str">
-        <v>shared umbrella with monks</v>
+        <v/>
       </c>
       <c r="N41" t="str">
-        <v>che chung ô cùng các nhà sư</v>
+        <v>Danh từ · Keyword</v>
       </c>
       <c r="O41" t="str">
-        <v>Ending</v>
+        <v>Từ nối · Logic word</v>
       </c>
       <c r="P41" t="str">
-        <v/>
+        <v>Cụm gợi hình · Fancy word</v>
       </c>
       <c r="Q41" t="str">
-        <v/>
+        <v>Tính từ · Ending</v>
       </c>
       <c r="R41" t="str">
         <v/>
@@ -2700,52 +2598,52 @@
         <v>3</v>
       </c>
       <c r="B42">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C42">
         <v>4</v>
       </c>
       <c r="D42" t="str">
-        <v>food court hunt</v>
+        <v>How long</v>
       </c>
       <c r="E42" t="str">
-        <v>công cuộc tìm kiếm khu ẩm thực</v>
+        <v>if</v>
       </c>
       <c r="F42" t="str">
-        <v>Keyword</v>
+        <v>green light</v>
       </c>
       <c r="G42" t="str">
-        <v>navigating towards the</v>
+        <v>smooth</v>
       </c>
       <c r="H42" t="str">
-        <v>dò dẫm bước về phía...</v>
+        <v/>
       </c>
       <c r="I42" t="str">
-        <v>Logic word</v>
+        <v>Bao lâu</v>
       </c>
       <c r="J42" t="str">
-        <v>bustling transit concourse</v>
+        <v>nếu</v>
       </c>
       <c r="K42" t="str">
-        <v>sảnh trung chuyển nhộn nhịp</v>
+        <v>bật đèn xanh</v>
       </c>
       <c r="L42" t="str">
-        <v>Fancy word</v>
+        <v>trơn tru</v>
       </c>
       <c r="M42" t="str">
-        <v>ordered steaming noodle soup</v>
+        <v/>
       </c>
       <c r="N42" t="str">
-        <v>gọi ngay bát mì nóng hổi</v>
+        <v>Cụm nghi vấn · WH word</v>
       </c>
       <c r="O42" t="str">
-        <v>Ending</v>
+        <v>Từ nối · Logic word</v>
       </c>
       <c r="P42" t="str">
-        <v/>
+        <v>Ẩn dụ · Fancy word</v>
       </c>
       <c r="Q42" t="str">
-        <v/>
+        <v>Tính từ · Ending</v>
       </c>
       <c r="R42" t="str">
         <v/>
@@ -2756,52 +2654,52 @@
         <v>3</v>
       </c>
       <c r="B43">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C43">
         <v>4</v>
       </c>
       <c r="D43" t="str">
-        <v>foreign socket adapter</v>
+        <v>budget airline</v>
       </c>
       <c r="E43" t="str">
-        <v>đầu chuyển ổ cắm điện nước ngoài</v>
+        <v>nevertheless</v>
       </c>
       <c r="F43" t="str">
-        <v>Keyword</v>
+        <v>hidden cost</v>
       </c>
       <c r="G43" t="str">
-        <v>struggling without a</v>
+        <v>pricey</v>
       </c>
       <c r="H43" t="str">
-        <v>chật vật xoay sở vì thiếu...</v>
+        <v/>
       </c>
       <c r="I43" t="str">
-        <v>Logic word</v>
+        <v>hãng bay giá rẻ</v>
       </c>
       <c r="J43" t="str">
-        <v>universal power converter</v>
+        <v>dù vậy</v>
       </c>
       <c r="K43" t="str">
-        <v>bộ chuyển đổi phích cắm đa năng</v>
+        <v>chi phí ngầm</v>
       </c>
       <c r="L43" t="str">
-        <v>Fancy word</v>
+        <v>đắt đỏ</v>
       </c>
       <c r="M43" t="str">
-        <v>borrowed one from reception</v>
+        <v/>
       </c>
       <c r="N43" t="str">
-        <v>mượn tạm một cái từ quầy tiếp tân</v>
+        <v>Danh từ · Keyword</v>
       </c>
       <c r="O43" t="str">
-        <v>Ending</v>
+        <v>Từ nối · Logic word</v>
       </c>
       <c r="P43" t="str">
-        <v/>
+        <v>Ẩn dụ · Fancy word</v>
       </c>
       <c r="Q43" t="str">
-        <v/>
+        <v>Tính từ · Ending</v>
       </c>
       <c r="R43" t="str">
         <v/>
@@ -2812,52 +2710,52 @@
         <v>3</v>
       </c>
       <c r="B44">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C44">
         <v>4</v>
       </c>
       <c r="D44" t="str">
-        <v>loose change pouch</v>
+        <v>commuter train</v>
       </c>
       <c r="E44" t="str">
-        <v>túi vải nhỏ đựng tiền lẻ</v>
+        <v>before that</v>
       </c>
       <c r="F44" t="str">
-        <v>Keyword</v>
+        <v>rush hour</v>
       </c>
       <c r="G44" t="str">
-        <v>emptying out the</v>
+        <v>packed</v>
       </c>
       <c r="H44" t="str">
-        <v>dốc hết...</v>
+        <v/>
       </c>
       <c r="I44" t="str">
-        <v>Logic word</v>
+        <v>tàu trung chuyển</v>
       </c>
       <c r="J44" t="str">
-        <v>foreign metal currency</v>
+        <v>trước đó</v>
       </c>
       <c r="K44" t="str">
-        <v>tiền xu ngoại tệ lỉnh kỉnh</v>
+        <v>giờ cao điểm</v>
       </c>
       <c r="L44" t="str">
-        <v>Fancy word</v>
+        <v>chật ních</v>
       </c>
       <c r="M44" t="str">
-        <v>bought chilled herbal drink</v>
+        <v/>
       </c>
       <c r="N44" t="str">
-        <v>mua lon nước sâm ướp lạnh giải khát</v>
+        <v>Danh từ · Keyword</v>
       </c>
       <c r="O44" t="str">
-        <v>Ending</v>
+        <v>Từ nối · Logic word</v>
       </c>
       <c r="P44" t="str">
-        <v/>
+        <v>Cụm gợi hình · Fancy word</v>
       </c>
       <c r="Q44" t="str">
-        <v/>
+        <v>Tính từ · Ending</v>
       </c>
       <c r="R44" t="str">
         <v/>
@@ -2868,52 +2766,52 @@
         <v>3</v>
       </c>
       <c r="B45">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C45">
         <v>4</v>
       </c>
       <c r="D45" t="str">
-        <v>overnight transit</v>
+        <v>travel SIM</v>
       </c>
       <c r="E45" t="str">
-        <v>chuyến bay quá cảnh qua đêm</v>
+        <v>in addition</v>
       </c>
       <c r="F45" t="str">
-        <v>Keyword</v>
+        <v>game changer</v>
       </c>
       <c r="G45" t="str">
-        <v>enduring the</v>
+        <v>connected</v>
       </c>
       <c r="H45" t="str">
-        <v>chịu đựng...</v>
+        <v/>
       </c>
       <c r="I45" t="str">
-        <v>Logic word</v>
+        <v>SIM du lịch</v>
       </c>
       <c r="J45" t="str">
-        <v>freezing airport terminal</v>
+        <v>hơn nữa</v>
       </c>
       <c r="K45" t="str">
-        <v>nhà ga sân bay lạnh buốt người</v>
+        <v>bước đột phá</v>
       </c>
       <c r="L45" t="str">
-        <v>Fancy word</v>
+        <v>thông suốt</v>
       </c>
       <c r="M45" t="str">
-        <v>wrapped tight in jacket</v>
+        <v/>
       </c>
       <c r="N45" t="str">
-        <v>quấn chặt mình trong chiếc áo khoác dày</v>
+        <v>Danh từ · Keyword</v>
       </c>
       <c r="O45" t="str">
-        <v>Ending</v>
+        <v>Từ nối · Logic word</v>
       </c>
       <c r="P45" t="str">
-        <v/>
+        <v>Ẩn dụ · Fancy word</v>
       </c>
       <c r="Q45" t="str">
-        <v/>
+        <v>Tính từ · Ending</v>
       </c>
       <c r="R45" t="str">
         <v/>
@@ -2924,52 +2822,52 @@
         <v>3</v>
       </c>
       <c r="B46">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C46">
         <v>4</v>
       </c>
       <c r="D46" t="str">
-        <v>lost destination shuttle</v>
+        <v>Where to go</v>
       </c>
       <c r="E46" t="str">
-        <v>chuyến xe buýt trung chuyển bị lạc</v>
+        <v>next</v>
       </c>
       <c r="F46" t="str">
-        <v>Keyword</v>
+        <v>hidden gem</v>
       </c>
       <c r="G46" t="str">
-        <v>confused inside the</v>
+        <v>breathtaking</v>
       </c>
       <c r="H46" t="str">
-        <v>hoang mang giữa...</v>
+        <v/>
       </c>
       <c r="I46" t="str">
-        <v>Logic word</v>
+        <v>Đi đâu bây giờ</v>
       </c>
       <c r="J46" t="str">
-        <v>labyrinthine arrival corridor</v>
+        <v>tiếp theo</v>
       </c>
       <c r="K46" t="str">
-        <v>hành lang ga đến như mê cung</v>
+        <v>viên ngọc ẩn</v>
       </c>
       <c r="L46" t="str">
-        <v>Fancy word</v>
+        <v>tuyệt đẹp</v>
       </c>
       <c r="M46" t="str">
-        <v>followed airline ground staff</v>
+        <v/>
       </c>
       <c r="N46" t="str">
-        <v>bám theo nhân viên mặt đất dẫn đường</v>
+        <v>Cụm nghi vấn · WH word</v>
       </c>
       <c r="O46" t="str">
-        <v>Ending</v>
+        <v>Từ nối · Logic word</v>
       </c>
       <c r="P46" t="str">
-        <v/>
+        <v>Ẩn dụ · Fancy word</v>
       </c>
       <c r="Q46" t="str">
-        <v/>
+        <v>Tính từ · Ending</v>
       </c>
       <c r="R46" t="str">
         <v/>
@@ -2977,114 +2875,114 @@
     </row>
     <row r="47">
       <c r="A47">
+        <v>3</v>
+      </c>
+      <c r="B47">
+        <v>14</v>
+      </c>
+      <c r="C47">
         <v>4</v>
       </c>
-      <c r="B47">
-        <v>1</v>
-      </c>
-      <c r="C47">
-        <v>5</v>
-      </c>
       <c r="D47" t="str">
-        <v>Just so you know</v>
+        <v>emergency exit</v>
       </c>
       <c r="E47" t="str">
-        <v>nói trước cho bạn biết là</v>
+        <v>for that reason</v>
       </c>
       <c r="F47" t="str">
-        <v>Intro</v>
+        <v>watchful eye</v>
       </c>
       <c r="G47" t="str">
-        <v>customs interrogation</v>
+        <v>alert</v>
       </c>
       <c r="H47" t="str">
-        <v>việc hải quan tra hỏi</v>
+        <v/>
       </c>
       <c r="I47" t="str">
-        <v>Keyword</v>
+        <v>cửa thoát hiểm</v>
       </c>
       <c r="J47" t="str">
-        <v>became tense because</v>
+        <v>chính vì thế</v>
       </c>
       <c r="K47" t="str">
-        <v>trở nên căng thẳng do...</v>
+        <v>ánh mắt quan sát</v>
       </c>
       <c r="L47" t="str">
-        <v>Logic word</v>
+        <v>cảnh giác</v>
       </c>
       <c r="M47" t="str">
-        <v>suspicious baggage contents</v>
+        <v/>
       </c>
       <c r="N47" t="str">
-        <v>kiện hành lý có dấu hiệu nghi vấn</v>
+        <v>Danh từ · Keyword</v>
       </c>
       <c r="O47" t="str">
-        <v>Fancy word</v>
+        <v>Từ nối · Logic word</v>
       </c>
       <c r="P47" t="str">
-        <v>opened bags for inspection</v>
+        <v>Ẩn dụ · Fancy word</v>
       </c>
       <c r="Q47" t="str">
-        <v>đã phải mở toang vali cho họ kiểm tra</v>
+        <v>Tính từ · Ending</v>
       </c>
       <c r="R47" t="str">
-        <v>Ending</v>
+        <v/>
       </c>
     </row>
     <row r="48">
       <c r="A48">
+        <v>3</v>
+      </c>
+      <c r="B48">
+        <v>15</v>
+      </c>
+      <c r="C48">
         <v>4</v>
       </c>
-      <c r="B48">
-        <v>2</v>
-      </c>
-      <c r="C48">
-        <v>5</v>
-      </c>
       <c r="D48" t="str">
-        <v>It seems that</v>
+        <v>night market</v>
       </c>
       <c r="E48" t="str">
-        <v>hình như là</v>
+        <v>then</v>
       </c>
       <c r="F48" t="str">
-        <v>Intro</v>
+        <v>food heaven</v>
       </c>
       <c r="G48" t="str">
-        <v>cheap flip-flops</v>
+        <v>bustling</v>
       </c>
       <c r="H48" t="str">
-        <v>đôi dép lào giá rẻ</v>
+        <v/>
       </c>
       <c r="I48" t="str">
-        <v>Keyword</v>
+        <v>khu chợ đêm</v>
       </c>
       <c r="J48" t="str">
-        <v>snapped suddenly while</v>
+        <v>sau đó</v>
       </c>
       <c r="K48" t="str">
-        <v>bị đứt phựt khi đang...</v>
+        <v>thiên đường món ngon</v>
       </c>
       <c r="L48" t="str">
-        <v>Logic word</v>
+        <v>nhộn nhịp</v>
       </c>
       <c r="M48" t="str">
-        <v>sprinting through terminal</v>
+        <v/>
       </c>
       <c r="N48" t="str">
-        <v>chạy thục mạng qua nhà ga vắng</v>
+        <v>Danh từ · Keyword</v>
       </c>
       <c r="O48" t="str">
-        <v>Fancy word</v>
+        <v>Từ nối · Logic word</v>
       </c>
       <c r="P48" t="str">
-        <v>barely caught departing flight</v>
+        <v>Ẩn dụ · Fancy word</v>
       </c>
       <c r="Q48" t="str">
-        <v>vừa vặn kịp bước lên chuyến bay</v>
+        <v>Tính từ · Ending</v>
       </c>
       <c r="R48" t="str">
-        <v>Ending</v>
+        <v/>
       </c>
     </row>
     <row r="49">
@@ -3092,55 +2990,55 @@
         <v>4</v>
       </c>
       <c r="B49">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C49">
         <v>5</v>
       </c>
       <c r="D49" t="str">
-        <v>No wonder</v>
+        <v>Just so you know</v>
       </c>
       <c r="E49" t="str">
-        <v>hèn chi / chả trách</v>
+        <v>boarding gate</v>
       </c>
       <c r="F49" t="str">
-        <v>Intro</v>
+        <v>meanwhile</v>
       </c>
       <c r="G49" t="str">
-        <v>wandering tourist soul</v>
+        <v>final call</v>
       </c>
       <c r="H49" t="str">
-        <v>kẻ du lịch lạc bước</v>
+        <v>hurry</v>
       </c>
       <c r="I49" t="str">
-        <v>Keyword</v>
+        <v>Nói trước cho bạn hay</v>
       </c>
       <c r="J49" t="str">
-        <v>felt exhausted after</v>
+        <v>cửa lên tàu bay</v>
       </c>
       <c r="K49" t="str">
-        <v>thấm mệt sau khi...</v>
+        <v>đồng thời</v>
       </c>
       <c r="L49" t="str">
-        <v>Logic word</v>
+        <v>hiệu lệnh cuối</v>
       </c>
       <c r="M49" t="str">
-        <v>aimless urban detour</v>
+        <v>khẩn trương</v>
       </c>
       <c r="N49" t="str">
-        <v>chuyến đi vòng quanh phố không định hướng</v>
+        <v>Cụm mào đầu · Intro</v>
       </c>
       <c r="O49" t="str">
-        <v>Fancy word</v>
+        <v>Danh từ · Keyword</v>
       </c>
       <c r="P49" t="str">
-        <v>collapsed onto hotel bed</v>
+        <v>Từ nối · Logic word</v>
       </c>
       <c r="Q49" t="str">
-        <v>ngã vật xuống giường khách sạn</v>
+        <v>Cụm gợi hình · Fancy word</v>
       </c>
       <c r="R49" t="str">
-        <v>Ending</v>
+        <v>Động từ · Ending</v>
       </c>
     </row>
     <row r="50">
@@ -3148,55 +3046,55 @@
         <v>4</v>
       </c>
       <c r="B50">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C50">
         <v>5</v>
       </c>
       <c r="D50" t="str">
-        <v>What'd you mean</v>
+        <v>To tell you the truth</v>
       </c>
       <c r="E50" t="str">
-        <v>ý bạn là sao khi bảo</v>
+        <v>rough turbulence</v>
       </c>
       <c r="F50" t="str">
-        <v>Intro</v>
+        <v>while</v>
       </c>
       <c r="G50" t="str">
-        <v>missing boarding pass</v>
+        <v>roller coaster</v>
       </c>
       <c r="H50" t="str">
-        <v>thẻ lên tàu bay biến mất</v>
+        <v>scary</v>
       </c>
       <c r="I50" t="str">
-        <v>Keyword</v>
+        <v>Thật lòng mà nói</v>
       </c>
       <c r="J50" t="str">
-        <v>was swallowed inside</v>
+        <v>nhiễu động dữ dội</v>
       </c>
       <c r="K50" t="str">
-        <v>đã bị kẹt sâu trong...</v>
+        <v>trong khi</v>
       </c>
       <c r="L50" t="str">
-        <v>Logic word</v>
+        <v>tàu lượn rung giật</v>
       </c>
       <c r="M50" t="str">
-        <v>faulty automated kiosk</v>
+        <v>đáng sợ</v>
       </c>
       <c r="N50" t="str">
-        <v>máy in vé tự động bị lỗi</v>
+        <v>Cụm mào đầu · Intro</v>
       </c>
       <c r="O50" t="str">
-        <v>Fancy word</v>
+        <v>Danh từ · Keyword</v>
       </c>
       <c r="P50" t="str">
-        <v>called airline duty officer</v>
+        <v>Từ nối · Logic word</v>
       </c>
       <c r="Q50" t="str">
-        <v>phải gọi nhân viên trực quầy ra xử lý</v>
+        <v>Ẩn dụ · Fancy word</v>
       </c>
       <c r="R50" t="str">
-        <v>Ending</v>
+        <v>Tính từ · Ending</v>
       </c>
     </row>
     <row r="51">
@@ -3204,55 +3102,55 @@
         <v>4</v>
       </c>
       <c r="B51">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C51">
         <v>5</v>
       </c>
       <c r="D51" t="str">
-        <v>Forget about it</v>
+        <v>It seems that</v>
       </c>
       <c r="E51" t="str">
-        <v>thôi bỏ qua chuyện đó đi</v>
+        <v>customs officer</v>
       </c>
       <c r="F51" t="str">
-        <v>Intro</v>
+        <v>however</v>
       </c>
       <c r="G51" t="str">
-        <v>overpriced airport snack</v>
+        <v>eagle eye</v>
       </c>
       <c r="H51" t="str">
-        <v>món ăn vặt đắt đỏ ở sân bay</v>
+        <v>thorough</v>
       </c>
       <c r="I51" t="str">
-        <v>Keyword</v>
+        <v>Có vẻ như là</v>
       </c>
       <c r="J51" t="str">
-        <v>wasted money unless</v>
+        <v>nhân viên hải quan</v>
       </c>
       <c r="K51" t="str">
-        <v>chỉ tổ phí tiền trừ khi...</v>
+        <v>tuy nhiên</v>
       </c>
       <c r="L51" t="str">
-        <v>Logic word</v>
+        <v>mắt đại bàng</v>
       </c>
       <c r="M51" t="str">
-        <v>famished starving traveler</v>
+        <v>kỹ lưỡng</v>
       </c>
       <c r="N51" t="str">
-        <v>người lữ hành đói lả ruột gan</v>
+        <v>Cụm mào đầu · Intro</v>
       </c>
       <c r="O51" t="str">
-        <v>Fancy word</v>
+        <v>Danh từ · Keyword</v>
       </c>
       <c r="P51" t="str">
-        <v>settles for stale sandwich</v>
+        <v>Từ nối · Logic word</v>
       </c>
       <c r="Q51" t="str">
-        <v>chấp nhận ăn tạm ổ bánh mì nguội</v>
+        <v>Ẩn dụ · Fancy word</v>
       </c>
       <c r="R51" t="str">
-        <v>Ending</v>
+        <v>Tính từ · Ending</v>
       </c>
     </row>
     <row r="52">
@@ -3260,55 +3158,55 @@
         <v>4</v>
       </c>
       <c r="B52">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C52">
         <v>5</v>
       </c>
       <c r="D52" t="str">
-        <v>Seriously now</v>
+        <v>As far as I know</v>
       </c>
       <c r="E52" t="str">
-        <v>nói nghiêm túc nhé</v>
+        <v>entry visa</v>
       </c>
       <c r="F52" t="str">
-        <v>Intro</v>
+        <v>otherwise</v>
       </c>
       <c r="G52" t="str">
-        <v>luggage trolley collision</v>
+        <v>red tape</v>
       </c>
       <c r="H52" t="str">
-        <v>cú va quẹt xe đẩy hành lý</v>
+        <v>delayed</v>
       </c>
       <c r="I52" t="str">
-        <v>Keyword</v>
+        <v>Theo chỗ tôi biết</v>
       </c>
       <c r="J52" t="str">
-        <v>happened solely due to</v>
+        <v>thị thực nhập cảnh</v>
       </c>
       <c r="K52" t="str">
-        <v>xảy ra chỉ vì...</v>
+        <v>nếu không</v>
       </c>
       <c r="L52" t="str">
-        <v>Logic word</v>
+        <v>thủ tục quan liêu</v>
       </c>
       <c r="M52" t="str">
-        <v>reckless crowded maneuvering</v>
+        <v>bị ách lại</v>
       </c>
       <c r="N52" t="str">
-        <v>cú luồn lách bất cẩn giữa đám đông</v>
+        <v>Cụm mào đầu · Intro</v>
       </c>
       <c r="O52" t="str">
-        <v>Fancy word</v>
+        <v>Danh từ · Keyword</v>
       </c>
       <c r="P52" t="str">
-        <v>scattered souvenirs everywhere</v>
+        <v>Từ nối · Logic word</v>
       </c>
       <c r="Q52" t="str">
-        <v>làm quà lưu niệm rơi vãi khắp sàn</v>
+        <v>Ẩn dụ · Fancy word</v>
       </c>
       <c r="R52" t="str">
-        <v>Ending</v>
+        <v>Tính từ · Ending</v>
       </c>
     </row>
     <row r="53">
@@ -3316,55 +3214,55 @@
         <v>4</v>
       </c>
       <c r="B53">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C53">
         <v>5</v>
       </c>
       <c r="D53" t="str">
-        <v>How come you</v>
+        <v>Believe it or not</v>
       </c>
       <c r="E53" t="str">
-        <v>sao bạn lại có thể</v>
+        <v>baggage carousel</v>
       </c>
       <c r="F53" t="str">
-        <v>Intro</v>
+        <v>eventually</v>
       </c>
       <c r="G53" t="str">
-        <v>packed huge rice cooker</v>
+        <v>dead end</v>
       </c>
       <c r="H53" t="str">
-        <v>nhét nguyên chiếc nồi cơm điện to</v>
+        <v>jammed</v>
       </c>
       <c r="I53" t="str">
-        <v>Keyword</v>
+        <v>Tin hay không tùy bạn</v>
       </c>
       <c r="J53" t="str">
-        <v>inside carry-on before</v>
+        <v>băng chuyền hành lý</v>
       </c>
       <c r="K53" t="str">
-        <v>vào hành lý xách tay trước khi...</v>
+        <v>sau cùng</v>
       </c>
       <c r="L53" t="str">
-        <v>Logic word</v>
+        <v>chỗ kẹt nghẽn</v>
       </c>
       <c r="M53" t="str">
-        <v>strict security scan</v>
+        <v>bị kẹt cứng</v>
       </c>
       <c r="N53" t="str">
-        <v>khâu kiểm tra an ninh nghiêm ngặt</v>
+        <v>Cụm mào đầu · Intro</v>
       </c>
       <c r="O53" t="str">
-        <v>Fancy word</v>
+        <v>Danh từ · Keyword</v>
       </c>
       <c r="P53" t="str">
-        <v>aroused total officer suspicion</v>
+        <v>Từ nối · Logic word</v>
       </c>
       <c r="Q53" t="str">
-        <v>khiến nhân viên hải quan nghi ngờ ngay</v>
+        <v>Ẩn dụ · Fancy word</v>
       </c>
       <c r="R53" t="str">
-        <v>Ending</v>
+        <v>Tính từ · Ending</v>
       </c>
     </row>
     <row r="54">
@@ -3372,55 +3270,55 @@
         <v>4</v>
       </c>
       <c r="B54">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C54">
         <v>5</v>
       </c>
       <c r="D54" t="str">
-        <v>Any chance that</v>
+        <v>From my perspective</v>
       </c>
       <c r="E54" t="str">
-        <v>liệu có khả năng nào</v>
+        <v>sleeping pod</v>
       </c>
       <c r="F54" t="str">
-        <v>Intro</v>
+        <v>in addition</v>
       </c>
       <c r="G54" t="str">
-        <v>flight departure time</v>
+        <v>godsend</v>
       </c>
       <c r="H54" t="str">
-        <v>giờ cất cánh chuyến bay</v>
+        <v>comfortable</v>
       </c>
       <c r="I54" t="str">
-        <v>Keyword</v>
+        <v>Theo góc nhìn của tôi</v>
       </c>
       <c r="J54" t="str">
-        <v>gets postponed because of</v>
+        <v>buồng ngủ sân bay</v>
       </c>
       <c r="K54" t="str">
-        <v>bị dời lại vì...</v>
+        <v>hơn nữa</v>
       </c>
       <c r="L54" t="str">
-        <v>Logic word</v>
+        <v>món quà cứu cánh</v>
       </c>
       <c r="M54" t="str">
-        <v>approaching tropical typhoon</v>
+        <v>dễ chịu</v>
       </c>
       <c r="N54" t="str">
-        <v>cơn bão nhiệt đới đang tiến tới gần</v>
+        <v>Cụm mào đầu · Intro</v>
       </c>
       <c r="O54" t="str">
-        <v>Fancy word</v>
+        <v>Danh từ · Keyword</v>
       </c>
       <c r="P54" t="str">
-        <v>stranded us overnight inside</v>
+        <v>Từ nối · Logic word</v>
       </c>
       <c r="Q54" t="str">
-        <v>khiến cả nhóm kẹt lại qua đêm</v>
+        <v>Ẩn dụ · Fancy word</v>
       </c>
       <c r="R54" t="str">
-        <v>Ending</v>
+        <v>Tính từ · Ending</v>
       </c>
     </row>
     <row r="55">
@@ -3428,55 +3326,55 @@
         <v>4</v>
       </c>
       <c r="B55">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C55">
         <v>5</v>
       </c>
       <c r="D55" t="str">
-        <v>Sounds like a plan</v>
+        <v>In my opinion</v>
       </c>
       <c r="E55" t="str">
-        <v>nghe có vẻ là kế hoạch hay</v>
+        <v>street food</v>
       </c>
       <c r="F55" t="str">
-        <v>Intro</v>
+        <v>if</v>
       </c>
       <c r="G55" t="str">
-        <v>renting riverside tuktuk</v>
+        <v>gold mine</v>
       </c>
       <c r="H55" t="str">
-        <v>thuê xe tuktuk dọc bờ sông</v>
+        <v>authentic</v>
       </c>
       <c r="I55" t="str">
-        <v>Keyword</v>
+        <v>Theo quan điểm của tôi</v>
       </c>
       <c r="J55" t="str">
-        <v>so we can escape</v>
+        <v>món ăn đường phố</v>
       </c>
       <c r="K55" t="str">
-        <v>để chúng ta thoát khỏi...</v>
+        <v>nếu</v>
       </c>
       <c r="L55" t="str">
-        <v>Logic word</v>
+        <v>mỏ vàng ẩm thực</v>
       </c>
       <c r="M55" t="str">
-        <v>sweltering tropical heat</v>
+        <v>chuẩn vị</v>
       </c>
       <c r="N55" t="str">
-        <v>cái nóng oi ả nhiệt đới</v>
+        <v>Cụm mào đầu · Intro</v>
       </c>
       <c r="O55" t="str">
-        <v>Fancy word</v>
+        <v>Danh từ · Keyword</v>
       </c>
       <c r="P55" t="str">
-        <v>enjoy local night market</v>
+        <v>Từ nối · Logic word</v>
       </c>
       <c r="Q55" t="str">
-        <v>thỏa thích dạo chợ đêm bản địa</v>
+        <v>Ẩn dụ · Fancy word</v>
       </c>
       <c r="R55" t="str">
-        <v>Ending</v>
+        <v>Tính từ · Ending</v>
       </c>
     </row>
     <row r="56">
@@ -3484,55 +3382,55 @@
         <v>4</v>
       </c>
       <c r="B56">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C56">
         <v>5</v>
       </c>
       <c r="D56" t="str">
-        <v>Lemme tell you</v>
+        <v>Don't get me wrong</v>
       </c>
       <c r="E56" t="str">
-        <v>để tôi kể thẳng cho bạn</v>
+        <v>souvenir shop</v>
       </c>
       <c r="F56" t="str">
-        <v>Intro</v>
+        <v>nevertheless</v>
       </c>
       <c r="G56" t="str">
-        <v>allergic peanut reaction</v>
+        <v>tourist trap</v>
       </c>
       <c r="H56" t="str">
-        <v>cơn sốc dị ứng đậu phộng</v>
+        <v>pricey</v>
       </c>
       <c r="I56" t="str">
-        <v>Keyword</v>
+        <v>Đừng hiểu sai ý tôi</v>
       </c>
       <c r="J56" t="str">
-        <v>hit immediately after eating</v>
+        <v>cửa hàng lưu niệm</v>
       </c>
       <c r="K56" t="str">
-        <v>tái phát ngay sau khi ăn...</v>
+        <v>dù vậy</v>
       </c>
       <c r="L56" t="str">
-        <v>Logic word</v>
+        <v>cái bẫy du khách</v>
       </c>
       <c r="M56" t="str">
-        <v>mysterious street delicacy</v>
+        <v>đắt đỏ</v>
       </c>
       <c r="N56" t="str">
-        <v>món đặc sản đường phố lạ mắt</v>
+        <v>Cụm mào đầu · Intro</v>
       </c>
       <c r="O56" t="str">
-        <v>Fancy word</v>
+        <v>Danh từ · Keyword</v>
       </c>
       <c r="P56" t="str">
-        <v>rushed for medical help</v>
+        <v>Từ nối · Logic word</v>
       </c>
       <c r="Q56" t="str">
-        <v>phải hối hả đi tìm trạm sơ cứu</v>
+        <v>Ẩn dụ · Fancy word</v>
       </c>
       <c r="R56" t="str">
-        <v>Ending</v>
+        <v>Tính từ · Ending</v>
       </c>
     </row>
     <row r="57">
@@ -3540,55 +3438,55 @@
         <v>4</v>
       </c>
       <c r="B57">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C57">
         <v>5</v>
       </c>
       <c r="D57" t="str">
-        <v>No question that</v>
+        <v>As a matter of fact</v>
       </c>
       <c r="E57" t="str">
-        <v>không còn nghi ngờ gì nữa</v>
+        <v>flight attendant</v>
       </c>
       <c r="F57" t="str">
-        <v>Intro</v>
+        <v>therefore</v>
       </c>
       <c r="G57" t="str">
-        <v>ancient temple detour</v>
+        <v>lifesaver</v>
       </c>
       <c r="H57" t="str">
-        <v>chuyến rẽ vào thăm ngôi chùa cổ</v>
+        <v>supportive</v>
       </c>
       <c r="I57" t="str">
-        <v>Keyword</v>
+        <v>Thực tế là</v>
       </c>
       <c r="J57" t="str">
-        <v>became unforgettable once</v>
+        <v>tiếp viên hàng không</v>
       </c>
       <c r="K57" t="str">
-        <v>trở nên khó quên khi...</v>
+        <v>do đó</v>
       </c>
       <c r="L57" t="str">
-        <v>Logic word</v>
+        <v>vị cứu tinh</v>
       </c>
       <c r="M57" t="str">
-        <v>serene chanting monks</v>
+        <v>tận tình</v>
       </c>
       <c r="N57" t="str">
-        <v>những nhà sư tụng kinh thanh tịnh</v>
+        <v>Cụm mào đầu · Intro</v>
       </c>
       <c r="O57" t="str">
-        <v>Fancy word</v>
+        <v>Danh từ · Keyword</v>
       </c>
       <c r="P57" t="str">
-        <v>offered peaceful blessings</v>
+        <v>Từ nối · Logic word</v>
       </c>
       <c r="Q57" t="str">
-        <v>trao tặng lời chúc phúc an lành</v>
+        <v>Ẩn dụ · Fancy word</v>
       </c>
       <c r="R57" t="str">
-        <v>Ending</v>
+        <v>Tính từ · Ending</v>
       </c>
     </row>
     <row r="58">
@@ -3596,55 +3494,55 @@
         <v>4</v>
       </c>
       <c r="B58">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C58">
         <v>5</v>
       </c>
       <c r="D58" t="str">
-        <v>At that time</v>
+        <v>First of all</v>
       </c>
       <c r="E58" t="str">
-        <v>vào đúng thời điểm ấy</v>
+        <v>medical insurance</v>
       </c>
       <c r="F58" t="str">
-        <v>Intro</v>
+        <v>before that</v>
       </c>
       <c r="G58" t="str">
-        <v>lost hotel keycard</v>
+        <v>safety net</v>
       </c>
       <c r="H58" t="str">
-        <v>chiếc thẻ phòng khách sạn bị mất</v>
+        <v>vital</v>
       </c>
       <c r="I58" t="str">
-        <v>Keyword</v>
+        <v>Trước hết là</v>
       </c>
       <c r="J58" t="str">
-        <v>caused severe panic until</v>
+        <v>bảo hiểm y tế</v>
       </c>
       <c r="K58" t="str">
-        <v>gây nên một phen hoảng sợ cho tới khi...</v>
+        <v>trước đó</v>
       </c>
       <c r="L58" t="str">
-        <v>Logic word</v>
+        <v>lưới bảo hiểm an toàn</v>
       </c>
       <c r="M58" t="str">
-        <v>observant friendly housekeeper</v>
+        <v>sống còn</v>
       </c>
       <c r="N58" t="str">
-        <v>cô lao công tốt bụng và tinh mắt</v>
+        <v>Cụm mào đầu · Intro</v>
       </c>
       <c r="O58" t="str">
-        <v>Fancy word</v>
+        <v>Danh từ · Keyword</v>
       </c>
       <c r="P58" t="str">
-        <v>returned it with smile</v>
+        <v>Từ nối · Logic word</v>
       </c>
       <c r="Q58" t="str">
-        <v>trao trả lại với nụ cười tươi</v>
+        <v>Ẩn dụ · Fancy word</v>
       </c>
       <c r="R58" t="str">
-        <v>Ending</v>
+        <v>Tính từ · Ending</v>
       </c>
     </row>
     <row r="59">
@@ -3652,55 +3550,55 @@
         <v>4</v>
       </c>
       <c r="B59">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C59">
         <v>5</v>
       </c>
       <c r="D59" t="str">
-        <v>Just leave it</v>
+        <v>By the way</v>
       </c>
       <c r="E59" t="str">
-        <v>cứ để nguyên nó trên bàn</v>
+        <v>hotel reception</v>
       </c>
       <c r="F59" t="str">
-        <v>Intro</v>
+        <v>next</v>
       </c>
       <c r="G59" t="str">
-        <v>spare change coins</v>
+        <v>warm welcome</v>
       </c>
       <c r="H59" t="str">
-        <v>mấy đồng tiền xu lẻ thừa</v>
+        <v>hospitable</v>
       </c>
       <c r="I59" t="str">
-        <v>Keyword</v>
+        <v>Nhân tiện đây</v>
       </c>
       <c r="J59" t="str">
-        <v>intended specifically for</v>
+        <v>tiếp tân khách sạn</v>
       </c>
       <c r="K59" t="str">
-        <v>để dành riêng cho...</v>
+        <v>tiếp theo</v>
       </c>
       <c r="L59" t="str">
-        <v>Logic word</v>
+        <v>chào đón ấm áp</v>
       </c>
       <c r="M59" t="str">
-        <v>generous hotel tip</v>
+        <v>hiếu khách</v>
       </c>
       <c r="N59" t="str">
-        <v>khoản tiền boa xứng đáng cho khách sạn</v>
+        <v>Cụm mào đầu · Intro</v>
       </c>
       <c r="O59" t="str">
-        <v>Fancy word</v>
+        <v>Danh từ · Keyword</v>
       </c>
       <c r="P59" t="str">
-        <v>before checking out early</v>
+        <v>Từ nối · Logic word</v>
       </c>
       <c r="Q59" t="str">
-        <v>trước khi làm thủ tục trả phòng sớm</v>
+        <v>Cụm gợi hình · Fancy word</v>
       </c>
       <c r="R59" t="str">
-        <v>Ending</v>
+        <v>Tính từ · Ending</v>
       </c>
     </row>
     <row r="60">
@@ -3708,55 +3606,55 @@
         <v>4</v>
       </c>
       <c r="B60">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C60">
         <v>5</v>
       </c>
       <c r="D60" t="str">
-        <v>It appears that</v>
+        <v>Honestly speaking</v>
       </c>
       <c r="E60" t="str">
-        <v>có vẻ như là</v>
+        <v>overweight luggage</v>
       </c>
       <c r="F60" t="str">
-        <v>Intro</v>
+        <v>in other words</v>
       </c>
       <c r="G60" t="str">
-        <v>unfamiliar transit terminal</v>
+        <v>money pit</v>
       </c>
       <c r="H60" t="str">
-        <v>nhà ga trung chuyển xa lạ</v>
+        <v>costly</v>
       </c>
       <c r="I60" t="str">
-        <v>Keyword</v>
+        <v>Thành thật mà nói</v>
       </c>
       <c r="J60" t="str">
-        <v>confused passengers due to</v>
+        <v>hành lý quá cước</v>
       </c>
       <c r="K60" t="str">
-        <v>làm hành khách bối rối bởi...</v>
+        <v>nói cách khác</v>
       </c>
       <c r="L60" t="str">
-        <v>Logic word</v>
+        <v>hố ngốn tiền</v>
       </c>
       <c r="M60" t="str">
-        <v>abrupt gate relocation</v>
+        <v>hao tốn</v>
       </c>
       <c r="N60" t="str">
-        <v>sự thay đổi cổng bay đột ngột</v>
+        <v>Cụm mào đầu · Intro</v>
       </c>
       <c r="O60" t="str">
-        <v>Fancy word</v>
+        <v>Danh từ · Keyword</v>
       </c>
       <c r="P60" t="str">
-        <v>forced crowd to sprint</v>
+        <v>Từ nối · Logic word</v>
       </c>
       <c r="Q60" t="str">
-        <v>khiến đám đông phải chạy đua vội vã</v>
+        <v>Ẩn dụ · Fancy word</v>
       </c>
       <c r="R60" t="str">
-        <v>Ending</v>
+        <v>Tính từ · Ending</v>
       </c>
     </row>
     <row r="61">
@@ -3764,60 +3662,172 @@
         <v>4</v>
       </c>
       <c r="B61">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C61">
         <v>5</v>
       </c>
       <c r="D61" t="str">
-        <v>For what reason</v>
+        <v>Keep in mind</v>
       </c>
       <c r="E61" t="str">
-        <v>vì lý do gì mà</v>
+        <v>meter taxi</v>
       </c>
       <c r="F61" t="str">
-        <v>Intro</v>
+        <v>as long as</v>
       </c>
       <c r="G61" t="str">
-        <v>bulky winter sleeping bag</v>
+        <v>fair play</v>
       </c>
       <c r="H61" t="str">
-        <v>chiếc túi ngủ mùa đông cồng kềnh</v>
+        <v>honest</v>
       </c>
       <c r="I61" t="str">
-        <v>Keyword</v>
+        <v>Hãy luôn ghi nhớ</v>
       </c>
       <c r="J61" t="str">
-        <v>was brought along when</v>
+        <v>taxi có đồng hồ</v>
       </c>
       <c r="K61" t="str">
-        <v>lại được mang theo trong khi...</v>
+        <v>miễn là</v>
       </c>
       <c r="L61" t="str">
-        <v>Logic word</v>
+        <v>chơi đẹp minh bạch</v>
       </c>
       <c r="M61" t="str">
-        <v>sweltering tropical island</v>
+        <v>trung thực</v>
       </c>
       <c r="N61" t="str">
-        <v>hòn đảo nhiệt đới nắng gắt</v>
+        <v>Cụm mào đầu · Intro</v>
       </c>
       <c r="O61" t="str">
-        <v>Fancy word</v>
+        <v>Danh từ · Keyword</v>
       </c>
       <c r="P61" t="str">
-        <v>only requires light flip-flops</v>
+        <v>Từ nối · Logic word</v>
       </c>
       <c r="Q61" t="str">
-        <v>chỉ cần một đôi dép lào nhẹ tênh</v>
+        <v>Ẩn dụ · Fancy word</v>
       </c>
       <c r="R61" t="str">
-        <v>Ending</v>
+        <v>Tính từ · Ending</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62">
+        <v>4</v>
+      </c>
+      <c r="B62">
+        <v>14</v>
+      </c>
+      <c r="C62">
+        <v>5</v>
+      </c>
+      <c r="D62" t="str">
+        <v>You can bet that</v>
+      </c>
+      <c r="E62" t="str">
+        <v>ocean sunrise</v>
+      </c>
+      <c r="F62" t="str">
+        <v>then</v>
+      </c>
+      <c r="G62" t="str">
+        <v>postcard view</v>
+      </c>
+      <c r="H62" t="str">
+        <v>stunning</v>
+      </c>
+      <c r="I62" t="str">
+        <v>Bạn cứ yên tâm rằng</v>
+      </c>
+      <c r="J62" t="str">
+        <v>bình minh biển</v>
+      </c>
+      <c r="K62" t="str">
+        <v>sau đó</v>
+      </c>
+      <c r="L62" t="str">
+        <v>khung cảnh như tranh</v>
+      </c>
+      <c r="M62" t="str">
+        <v>đẹp ngỡ ngàng</v>
+      </c>
+      <c r="N62" t="str">
+        <v>Cụm mào đầu · Intro</v>
+      </c>
+      <c r="O62" t="str">
+        <v>Danh từ · Keyword</v>
+      </c>
+      <c r="P62" t="str">
+        <v>Từ nối · Logic word</v>
+      </c>
+      <c r="Q62" t="str">
+        <v>Cụm gợi hình · Fancy word</v>
+      </c>
+      <c r="R62" t="str">
+        <v>Tính từ · Ending</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63">
+        <v>4</v>
+      </c>
+      <c r="B63">
+        <v>15</v>
+      </c>
+      <c r="C63">
+        <v>5</v>
+      </c>
+      <c r="D63" t="str">
+        <v>All things considered</v>
+      </c>
+      <c r="E63" t="str">
+        <v>solo trip</v>
+      </c>
+      <c r="F63" t="str">
+        <v>finally</v>
+      </c>
+      <c r="G63" t="str">
+        <v>eye opener</v>
+      </c>
+      <c r="H63" t="str">
+        <v>unforgettable</v>
+      </c>
+      <c r="I63" t="str">
+        <v>Cân nhắc mọi mặt</v>
+      </c>
+      <c r="J63" t="str">
+        <v>chuyến du hành độc hành</v>
+      </c>
+      <c r="K63" t="str">
+        <v>cuối cùng</v>
+      </c>
+      <c r="L63" t="str">
+        <v>trải nghiệm mở rộng tầm mắt</v>
+      </c>
+      <c r="M63" t="str">
+        <v>khó quên</v>
+      </c>
+      <c r="N63" t="str">
+        <v>Cụm mào đầu · Intro</v>
+      </c>
+      <c r="O63" t="str">
+        <v>Danh từ · Keyword</v>
+      </c>
+      <c r="P63" t="str">
+        <v>Từ nối · Logic word</v>
+      </c>
+      <c r="Q63" t="str">
+        <v>Ẩn dụ · Fancy word</v>
+      </c>
+      <c r="R63" t="str">
+        <v>Tính từ · Ending</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:R61"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:R63"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(improv): enhance excel parser flexibility, add retry write safety, and align default package schemas
</commit_message>
<xml_diff>
--- a/public/data/Improv_Set_01_Wandering_Souls.xlsx
+++ b/public/data/Improv_Set_01_Wandering_Souls.xlsx
@@ -647,7 +647,7 @@
         <v>customs officer</v>
       </c>
       <c r="E7" t="str">
-        <v>check</v>
+        <v>passport</v>
       </c>
       <c r="F7" t="str">
         <v/>
@@ -662,7 +662,7 @@
         <v>nhân viên hải quan</v>
       </c>
       <c r="J7" t="str">
-        <v>kiểm tra</v>
+        <v>hộ chiếu</v>
       </c>
       <c r="K7" t="str">
         <v/>
@@ -677,7 +677,7 @@
         <v>Danh từ · Keyword</v>
       </c>
       <c r="O7" t="str">
-        <v>Động từ · Ending</v>
+        <v>Danh từ · Ending</v>
       </c>
       <c r="P7" t="str">
         <v/>
@@ -868,10 +868,10 @@
         <v>2</v>
       </c>
       <c r="D11" t="str">
-        <v>passport</v>
+        <v>suitcase</v>
       </c>
       <c r="E11" t="str">
-        <v>forget</v>
+        <v>lock</v>
       </c>
       <c r="F11" t="str">
         <v/>
@@ -883,10 +883,10 @@
         <v/>
       </c>
       <c r="I11" t="str">
-        <v>hộ chiếu</v>
+        <v>vali</v>
       </c>
       <c r="J11" t="str">
-        <v>quên</v>
+        <v>khóa</v>
       </c>
       <c r="K11" t="str">
         <v/>
@@ -924,10 +924,10 @@
         <v>2</v>
       </c>
       <c r="D12" t="str">
-        <v>suitcase</v>
+        <v>flip-flops</v>
       </c>
       <c r="E12" t="str">
-        <v>lock</v>
+        <v>beach trip</v>
       </c>
       <c r="F12" t="str">
         <v/>
@@ -939,10 +939,10 @@
         <v/>
       </c>
       <c r="I12" t="str">
-        <v>vali</v>
+        <v>dép lào</v>
       </c>
       <c r="J12" t="str">
-        <v>khóa</v>
+        <v>đi biển</v>
       </c>
       <c r="K12" t="str">
         <v/>
@@ -957,7 +957,7 @@
         <v>Danh từ · Keyword</v>
       </c>
       <c r="O12" t="str">
-        <v>Động từ · Ending</v>
+        <v>Danh từ · Ending</v>
       </c>
       <c r="P12" t="str">
         <v/>
@@ -980,10 +980,10 @@
         <v>2</v>
       </c>
       <c r="D13" t="str">
-        <v>flip-flops</v>
+        <v>boarding gate</v>
       </c>
       <c r="E13" t="str">
-        <v>beach trip</v>
+        <v>find</v>
       </c>
       <c r="F13" t="str">
         <v/>
@@ -995,10 +995,10 @@
         <v/>
       </c>
       <c r="I13" t="str">
-        <v>dép lào</v>
+        <v>cửa khởi hành</v>
       </c>
       <c r="J13" t="str">
-        <v>đi biển</v>
+        <v>tìm</v>
       </c>
       <c r="K13" t="str">
         <v/>
@@ -1013,7 +1013,7 @@
         <v>Danh từ · Keyword</v>
       </c>
       <c r="O13" t="str">
-        <v>Danh từ · Ending</v>
+        <v>Động từ · Ending</v>
       </c>
       <c r="P13" t="str">
         <v/>
@@ -1036,10 +1036,10 @@
         <v>2</v>
       </c>
       <c r="D14" t="str">
-        <v>boarding gate</v>
+        <v>snacks</v>
       </c>
       <c r="E14" t="str">
-        <v>find</v>
+        <v>bring along</v>
       </c>
       <c r="F14" t="str">
         <v/>
@@ -1051,10 +1051,10 @@
         <v/>
       </c>
       <c r="I14" t="str">
-        <v>cửa khởi hành</v>
+        <v>đồ ăn nhẹ</v>
       </c>
       <c r="J14" t="str">
-        <v>tìm</v>
+        <v>mang theo</v>
       </c>
       <c r="K14" t="str">
         <v/>
@@ -1092,10 +1092,10 @@
         <v>2</v>
       </c>
       <c r="D15" t="str">
-        <v>snacks</v>
+        <v>layover time</v>
       </c>
       <c r="E15" t="str">
-        <v>bring along</v>
+        <v>long</v>
       </c>
       <c r="F15" t="str">
         <v/>
@@ -1107,10 +1107,10 @@
         <v/>
       </c>
       <c r="I15" t="str">
-        <v>đồ ăn nhẹ</v>
+        <v>thời gian quá cảnh</v>
       </c>
       <c r="J15" t="str">
-        <v>mang theo</v>
+        <v>dài</v>
       </c>
       <c r="K15" t="str">
         <v/>
@@ -1125,7 +1125,7 @@
         <v>Danh từ · Keyword</v>
       </c>
       <c r="O15" t="str">
-        <v>Động từ · Ending</v>
+        <v>Tính từ · Ending</v>
       </c>
       <c r="P15" t="str">
         <v/>
@@ -1148,10 +1148,10 @@
         <v>2</v>
       </c>
       <c r="D16" t="str">
-        <v>layover time</v>
+        <v>taxi driver</v>
       </c>
       <c r="E16" t="str">
-        <v>long</v>
+        <v>friendly</v>
       </c>
       <c r="F16" t="str">
         <v/>
@@ -1163,10 +1163,10 @@
         <v/>
       </c>
       <c r="I16" t="str">
-        <v>thời gian quá cảnh</v>
+        <v>tài xế taxi</v>
       </c>
       <c r="J16" t="str">
-        <v>dài</v>
+        <v>thân thiện</v>
       </c>
       <c r="K16" t="str">
         <v/>
@@ -1204,10 +1204,10 @@
         <v>2</v>
       </c>
       <c r="D17" t="str">
-        <v>taxi driver</v>
+        <v>check-in counter</v>
       </c>
       <c r="E17" t="str">
-        <v>friendly</v>
+        <v>crowded</v>
       </c>
       <c r="F17" t="str">
         <v/>
@@ -1219,10 +1219,10 @@
         <v/>
       </c>
       <c r="I17" t="str">
-        <v>tài xế taxi</v>
+        <v>quầy thủ tục</v>
       </c>
       <c r="J17" t="str">
-        <v>thân thiện</v>
+        <v>đông đúc</v>
       </c>
       <c r="K17" t="str">
         <v/>
@@ -1260,10 +1260,10 @@
         <v>2</v>
       </c>
       <c r="D18" t="str">
-        <v>rice cooker</v>
+        <v>painkillers</v>
       </c>
       <c r="E18" t="str">
-        <v>cook rice</v>
+        <v>necessary</v>
       </c>
       <c r="F18" t="str">
         <v/>
@@ -1275,10 +1275,10 @@
         <v/>
       </c>
       <c r="I18" t="str">
-        <v>nồi cơm điện</v>
+        <v>thuốc giảm đau</v>
       </c>
       <c r="J18" t="str">
-        <v>nấu cơm</v>
+        <v>cần thiết</v>
       </c>
       <c r="K18" t="str">
         <v/>
@@ -1293,7 +1293,7 @@
         <v>Danh từ · Keyword</v>
       </c>
       <c r="O18" t="str">
-        <v>Động từ · Ending</v>
+        <v>Tính từ · Ending</v>
       </c>
       <c r="P18" t="str">
         <v/>
@@ -1316,13 +1316,13 @@
         <v>3</v>
       </c>
       <c r="D19" t="str">
-        <v>heavy luggage</v>
+        <v>boarding pass</v>
       </c>
       <c r="E19" t="str">
-        <v>therefore</v>
+        <v>in other words</v>
       </c>
       <c r="F19" t="str">
-        <v>exhausted</v>
+        <v>important</v>
       </c>
       <c r="G19" t="str">
         <v/>
@@ -1331,13 +1331,13 @@
         <v/>
       </c>
       <c r="I19" t="str">
-        <v>hành lý nặng</v>
+        <v>thẻ lên máy bay</v>
       </c>
       <c r="J19" t="str">
-        <v>do đó</v>
+        <v>nói cách khác</v>
       </c>
       <c r="K19" t="str">
-        <v>mệt lử</v>
+        <v>quan trọng</v>
       </c>
       <c r="L19" t="str">
         <v/>
@@ -1372,13 +1372,13 @@
         <v>3</v>
       </c>
       <c r="D20" t="str">
-        <v>passport renewal</v>
+        <v>check-in counter</v>
       </c>
       <c r="E20" t="str">
-        <v>before that</v>
+        <v>in addition</v>
       </c>
       <c r="F20" t="str">
-        <v>urgent</v>
+        <v>crowded</v>
       </c>
       <c r="G20" t="str">
         <v/>
@@ -1387,13 +1387,13 @@
         <v/>
       </c>
       <c r="I20" t="str">
-        <v>gia hạn hộ chiếu</v>
+        <v>quầy thủ tục</v>
       </c>
       <c r="J20" t="str">
-        <v>trước đó</v>
+        <v>hơn nữa</v>
       </c>
       <c r="K20" t="str">
-        <v>khẩn cấp</v>
+        <v>đông đúc</v>
       </c>
       <c r="L20" t="str">
         <v/>
@@ -1428,13 +1428,13 @@
         <v>3</v>
       </c>
       <c r="D21" t="str">
-        <v>flight delay</v>
+        <v>passport</v>
       </c>
       <c r="E21" t="str">
-        <v>meanwhile</v>
+        <v>before that</v>
       </c>
       <c r="F21" t="str">
-        <v>rest</v>
+        <v>safeguard</v>
       </c>
       <c r="G21" t="str">
         <v/>
@@ -1443,13 +1443,13 @@
         <v/>
       </c>
       <c r="I21" t="str">
-        <v>chuyến bay hoãn</v>
+        <v>hộ chiếu</v>
       </c>
       <c r="J21" t="str">
-        <v>đồng thời</v>
+        <v>trước đó</v>
       </c>
       <c r="K21" t="str">
-        <v>nghỉ ngơi</v>
+        <v>cất kỹ</v>
       </c>
       <c r="L21" t="str">
         <v/>
@@ -1484,13 +1484,13 @@
         <v>3</v>
       </c>
       <c r="D22" t="str">
-        <v>taxi fare</v>
+        <v>luggage cart</v>
       </c>
       <c r="E22" t="str">
-        <v>in addition</v>
+        <v>however</v>
       </c>
       <c r="F22" t="str">
-        <v>expensive</v>
+        <v>broken</v>
       </c>
       <c r="G22" t="str">
         <v/>
@@ -1499,13 +1499,13 @@
         <v/>
       </c>
       <c r="I22" t="str">
-        <v>tiền taxi</v>
+        <v>xe đẩy hành lý</v>
       </c>
       <c r="J22" t="str">
-        <v>hơn nữa</v>
+        <v>tuy nhiên</v>
       </c>
       <c r="K22" t="str">
-        <v>đắt đỏ</v>
+        <v>hỏng</v>
       </c>
       <c r="L22" t="str">
         <v/>
@@ -1540,13 +1540,13 @@
         <v>3</v>
       </c>
       <c r="D23" t="str">
-        <v>boarding gate</v>
+        <v>hotel</v>
       </c>
       <c r="E23" t="str">
-        <v>next</v>
+        <v>eventually</v>
       </c>
       <c r="F23" t="str">
-        <v>sprint</v>
+        <v>reschedule</v>
       </c>
       <c r="G23" t="str">
         <v/>
@@ -1555,13 +1555,13 @@
         <v/>
       </c>
       <c r="I23" t="str">
-        <v>cửa ra máy bay</v>
+        <v>khách sạn</v>
       </c>
       <c r="J23" t="str">
-        <v>tiếp theo</v>
+        <v>sau cùng</v>
       </c>
       <c r="K23" t="str">
-        <v>chạy nước rút</v>
+        <v>đổi lịch</v>
       </c>
       <c r="L23" t="str">
         <v/>
@@ -1596,13 +1596,13 @@
         <v>3</v>
       </c>
       <c r="D24" t="str">
-        <v>window seat</v>
+        <v>taxi fare</v>
       </c>
       <c r="E24" t="str">
-        <v>otherwise</v>
+        <v>therefore</v>
       </c>
       <c r="F24" t="str">
-        <v>cramped</v>
+        <v>reasonable</v>
       </c>
       <c r="G24" t="str">
         <v/>
@@ -1611,13 +1611,13 @@
         <v/>
       </c>
       <c r="I24" t="str">
-        <v>ghế cạnh cửa sổ</v>
+        <v>tiền taxi</v>
       </c>
       <c r="J24" t="str">
-        <v>nếu không</v>
+        <v>do đó</v>
       </c>
       <c r="K24" t="str">
-        <v>chật chội</v>
+        <v>hợp lý</v>
       </c>
       <c r="L24" t="str">
         <v/>
@@ -1652,13 +1652,13 @@
         <v>3</v>
       </c>
       <c r="D25" t="str">
-        <v>travel insurance</v>
+        <v>boarding gate</v>
       </c>
       <c r="E25" t="str">
-        <v>if</v>
+        <v>next</v>
       </c>
       <c r="F25" t="str">
-        <v>secure</v>
+        <v>sprint</v>
       </c>
       <c r="G25" t="str">
         <v/>
@@ -1667,13 +1667,13 @@
         <v/>
       </c>
       <c r="I25" t="str">
-        <v>bảo hiểm du lịch</v>
+        <v>cửa khởi hành</v>
       </c>
       <c r="J25" t="str">
-        <v>nếu</v>
+        <v>tiếp theo</v>
       </c>
       <c r="K25" t="str">
-        <v>an tâm</v>
+        <v>chạy nước rút</v>
       </c>
       <c r="L25" t="str">
         <v/>
@@ -1688,7 +1688,7 @@
         <v>Từ nối · Logic word</v>
       </c>
       <c r="P25" t="str">
-        <v>Tính từ · Ending</v>
+        <v>Động từ · Ending</v>
       </c>
       <c r="Q25" t="str">
         <v/>
@@ -1708,13 +1708,13 @@
         <v>3</v>
       </c>
       <c r="D26" t="str">
-        <v>broken wheel</v>
+        <v>travel insurance</v>
       </c>
       <c r="E26" t="str">
-        <v>nevertheless</v>
+        <v>if</v>
       </c>
       <c r="F26" t="str">
-        <v>manageable</v>
+        <v>secure</v>
       </c>
       <c r="G26" t="str">
         <v/>
@@ -1723,13 +1723,13 @@
         <v/>
       </c>
       <c r="I26" t="str">
-        <v>bánh xe bị gãy</v>
+        <v>bảo hiểm du lịch</v>
       </c>
       <c r="J26" t="str">
-        <v>dù vậy</v>
+        <v>nếu</v>
       </c>
       <c r="K26" t="str">
-        <v>xoay xở được</v>
+        <v>an tâm</v>
       </c>
       <c r="L26" t="str">
         <v/>
@@ -1764,13 +1764,13 @@
         <v>3</v>
       </c>
       <c r="D27" t="str">
-        <v>foreign currency</v>
+        <v>flight delay</v>
       </c>
       <c r="E27" t="str">
-        <v>in other words</v>
+        <v>meanwhile</v>
       </c>
       <c r="F27" t="str">
-        <v>exchange</v>
+        <v>rest</v>
       </c>
       <c r="G27" t="str">
         <v/>
@@ -1779,13 +1779,13 @@
         <v/>
       </c>
       <c r="I27" t="str">
-        <v>ngoại tệ</v>
+        <v>chuyến bay hoãn</v>
       </c>
       <c r="J27" t="str">
-        <v>nói cách khác</v>
+        <v>đồng thời</v>
       </c>
       <c r="K27" t="str">
-        <v>đổi tiền</v>
+        <v>nghỉ ngơi</v>
       </c>
       <c r="L27" t="str">
         <v/>
@@ -1820,13 +1820,13 @@
         <v>3</v>
       </c>
       <c r="D28" t="str">
-        <v>hotel room</v>
+        <v>window seat</v>
       </c>
       <c r="E28" t="str">
-        <v>eventually</v>
+        <v>otherwise</v>
       </c>
       <c r="F28" t="str">
-        <v>confirmed</v>
+        <v>cramped</v>
       </c>
       <c r="G28" t="str">
         <v/>
@@ -1835,13 +1835,13 @@
         <v/>
       </c>
       <c r="I28" t="str">
-        <v>phòng khách sạn</v>
+        <v>ghế cạnh cửa sổ</v>
       </c>
       <c r="J28" t="str">
-        <v>sau cùng</v>
+        <v>nếu không</v>
       </c>
       <c r="K28" t="str">
-        <v>xác nhận</v>
+        <v>chật chội</v>
       </c>
       <c r="L28" t="str">
         <v/>
@@ -1876,13 +1876,13 @@
         <v>3</v>
       </c>
       <c r="D29" t="str">
-        <v>street market</v>
+        <v>foreign currency</v>
       </c>
       <c r="E29" t="str">
-        <v>however</v>
+        <v>for example</v>
       </c>
       <c r="F29" t="str">
-        <v>crowded</v>
+        <v>exchange</v>
       </c>
       <c r="G29" t="str">
         <v/>
@@ -1891,13 +1891,13 @@
         <v/>
       </c>
       <c r="I29" t="str">
-        <v>chợ đường phố</v>
+        <v>ngoại tệ</v>
       </c>
       <c r="J29" t="str">
-        <v>tuy nhiên</v>
+        <v>ví dụ</v>
       </c>
       <c r="K29" t="str">
-        <v>đông đúc</v>
+        <v>đổi tiền</v>
       </c>
       <c r="L29" t="str">
         <v/>
@@ -1912,7 +1912,7 @@
         <v>Từ nối · Logic word</v>
       </c>
       <c r="P29" t="str">
-        <v>Tính từ · Ending</v>
+        <v>Động từ · Ending</v>
       </c>
       <c r="Q29" t="str">
         <v/>
@@ -1932,13 +1932,13 @@
         <v>3</v>
       </c>
       <c r="D30" t="str">
-        <v>transit flight</v>
+        <v>broken wheel</v>
       </c>
       <c r="E30" t="str">
-        <v>as long as</v>
+        <v>nevertheless</v>
       </c>
       <c r="F30" t="str">
-        <v>on time</v>
+        <v>manageable</v>
       </c>
       <c r="G30" t="str">
         <v/>
@@ -1947,13 +1947,13 @@
         <v/>
       </c>
       <c r="I30" t="str">
-        <v>chuyến bay quá cảnh</v>
+        <v>bánh xe hỏng</v>
       </c>
       <c r="J30" t="str">
-        <v>miễn là</v>
+        <v>dù vậy</v>
       </c>
       <c r="K30" t="str">
-        <v>đúng giờ</v>
+        <v>xoay xở được</v>
       </c>
       <c r="L30" t="str">
         <v/>
@@ -1988,13 +1988,13 @@
         <v>3</v>
       </c>
       <c r="D31" t="str">
-        <v>power bank</v>
+        <v>transit flight</v>
       </c>
       <c r="E31" t="str">
-        <v>for example</v>
+        <v>as long as</v>
       </c>
       <c r="F31" t="str">
-        <v>essential</v>
+        <v>on time</v>
       </c>
       <c r="G31" t="str">
         <v/>
@@ -2003,13 +2003,13 @@
         <v/>
       </c>
       <c r="I31" t="str">
-        <v>sạc dự phòng</v>
+        <v>chuyến bay quá cảnh</v>
       </c>
       <c r="J31" t="str">
-        <v>ví dụ</v>
+        <v>miễn là</v>
       </c>
       <c r="K31" t="str">
-        <v>thiết yếu</v>
+        <v>đúng giờ</v>
       </c>
       <c r="L31" t="str">
         <v/>
@@ -2044,13 +2044,13 @@
         <v>3</v>
       </c>
       <c r="D32" t="str">
-        <v>sudden rain</v>
+        <v>power bank</v>
       </c>
       <c r="E32" t="str">
-        <v>then</v>
+        <v>besides</v>
       </c>
       <c r="F32" t="str">
-        <v>take shelter</v>
+        <v>essential</v>
       </c>
       <c r="G32" t="str">
         <v/>
@@ -2059,13 +2059,13 @@
         <v/>
       </c>
       <c r="I32" t="str">
-        <v>mưa bất chợt</v>
+        <v>sạc dự phòng</v>
       </c>
       <c r="J32" t="str">
-        <v>sau đó</v>
+        <v>ngoài ra</v>
       </c>
       <c r="K32" t="str">
-        <v>trú mưa</v>
+        <v>thiết yếu</v>
       </c>
       <c r="L32" t="str">
         <v/>
@@ -2080,7 +2080,7 @@
         <v>Từ nối · Logic word</v>
       </c>
       <c r="P32" t="str">
-        <v>Động từ · Ending</v>
+        <v>Tính từ · Ending</v>
       </c>
       <c r="Q32" t="str">
         <v/>
@@ -2103,10 +2103,10 @@
         <v>tour guide</v>
       </c>
       <c r="E33" t="str">
-        <v>besides</v>
+        <v>then</v>
       </c>
       <c r="F33" t="str">
-        <v>knowledgeable</v>
+        <v>gather</v>
       </c>
       <c r="G33" t="str">
         <v/>
@@ -2118,10 +2118,10 @@
         <v>hướng dẫn viên</v>
       </c>
       <c r="J33" t="str">
-        <v>ngoài ra</v>
+        <v>sau đó</v>
       </c>
       <c r="K33" t="str">
-        <v>am hiểu</v>
+        <v>tập trung</v>
       </c>
       <c r="L33" t="str">
         <v/>
@@ -2136,7 +2136,7 @@
         <v>Từ nối · Logic word</v>
       </c>
       <c r="P33" t="str">
-        <v>Tính từ · Ending</v>
+        <v>Động từ · Ending</v>
       </c>
       <c r="Q33" t="str">
         <v/>
@@ -2156,31 +2156,31 @@
         <v>4</v>
       </c>
       <c r="D34" t="str">
-        <v>customs check</v>
+        <v>air conditioner</v>
       </c>
       <c r="E34" t="str">
         <v>while</v>
       </c>
       <c r="F34" t="str">
-        <v>red flag</v>
+        <v>soft hum</v>
       </c>
       <c r="G34" t="str">
-        <v>strict</v>
+        <v>all night</v>
       </c>
       <c r="H34" t="str">
         <v/>
       </c>
       <c r="I34" t="str">
-        <v>kiểm tra hải quan</v>
+        <v>máy lạnh</v>
       </c>
       <c r="J34" t="str">
         <v>trong khi</v>
       </c>
       <c r="K34" t="str">
-        <v>dấu hiệu khả nghi</v>
+        <v>rì rì</v>
       </c>
       <c r="L34" t="str">
-        <v>nghiêm ngặt</v>
+        <v>suốt đêm</v>
       </c>
       <c r="M34" t="str">
         <v/>
@@ -2192,10 +2192,10 @@
         <v>Từ nối · Logic word</v>
       </c>
       <c r="P34" t="str">
-        <v>Ẩn dụ · Fancy word</v>
+        <v>Từ tượng thanh · Fancy word</v>
       </c>
       <c r="Q34" t="str">
-        <v>Tính từ · Ending</v>
+        <v>Trạng từ · Ending</v>
       </c>
       <c r="R34" t="str">
         <v/>
@@ -2212,31 +2212,31 @@
         <v>4</v>
       </c>
       <c r="D35" t="str">
-        <v>airport terminal</v>
+        <v>boarding gate</v>
       </c>
       <c r="E35" t="str">
-        <v>however</v>
+        <v>but</v>
       </c>
       <c r="F35" t="str">
-        <v>lifeline</v>
+        <v>rush</v>
       </c>
       <c r="G35" t="str">
-        <v>helpful</v>
+        <v>on time</v>
       </c>
       <c r="H35" t="str">
         <v/>
       </c>
       <c r="I35" t="str">
-        <v>nhà ga sân bay</v>
+        <v>cửa khởi hành</v>
       </c>
       <c r="J35" t="str">
-        <v>tuy nhiên</v>
+        <v>nhưng</v>
       </c>
       <c r="K35" t="str">
-        <v>phao cứu trợ</v>
+        <v>vội vã</v>
       </c>
       <c r="L35" t="str">
-        <v>hữu ích</v>
+        <v>kịp giờ</v>
       </c>
       <c r="M35" t="str">
         <v/>
@@ -2248,7 +2248,7 @@
         <v>Từ nối · Logic word</v>
       </c>
       <c r="P35" t="str">
-        <v>Ẩn dụ · Fancy word</v>
+        <v>Cụm gợi hình · Fancy word</v>
       </c>
       <c r="Q35" t="str">
         <v>Tính từ · Ending</v>
@@ -2268,43 +2268,43 @@
         <v>4</v>
       </c>
       <c r="D36" t="str">
-        <v>Which flight</v>
+        <v>luggage</v>
       </c>
       <c r="E36" t="str">
-        <v>otherwise</v>
+        <v>in contrast</v>
       </c>
       <c r="F36" t="str">
-        <v>last call</v>
+        <v>heavy burden</v>
       </c>
       <c r="G36" t="str">
-        <v>missed</v>
+        <v>tired</v>
       </c>
       <c r="H36" t="str">
         <v/>
       </c>
       <c r="I36" t="str">
-        <v>Chuyến bay nào</v>
+        <v>hành lý</v>
       </c>
       <c r="J36" t="str">
-        <v>nếu không</v>
+        <v>ngược lại</v>
       </c>
       <c r="K36" t="str">
-        <v>loa gọi chót</v>
+        <v>nặng trĩu</v>
       </c>
       <c r="L36" t="str">
-        <v>bị lỡ</v>
+        <v>mệt mỏi</v>
       </c>
       <c r="M36" t="str">
         <v/>
       </c>
       <c r="N36" t="str">
-        <v>Cụm nghi vấn · WH word</v>
+        <v>Danh từ · Keyword</v>
       </c>
       <c r="O36" t="str">
         <v>Từ nối · Logic word</v>
       </c>
       <c r="P36" t="str">
-        <v>Cụm gợi hình · Fancy word</v>
+        <v>Ẩn dụ · Fancy word</v>
       </c>
       <c r="Q36" t="str">
         <v>Tính từ · Ending</v>
@@ -2324,31 +2324,31 @@
         <v>4</v>
       </c>
       <c r="D37" t="str">
-        <v>lost baggage</v>
+        <v>customs check</v>
       </c>
       <c r="E37" t="str">
         <v>therefore</v>
       </c>
       <c r="F37" t="str">
-        <v>headache</v>
+        <v>red flag</v>
       </c>
       <c r="G37" t="str">
-        <v>stressful</v>
+        <v>strict</v>
       </c>
       <c r="H37" t="str">
         <v/>
       </c>
       <c r="I37" t="str">
-        <v>thất lạc hành lý</v>
+        <v>kiểm tra hải quan</v>
       </c>
       <c r="J37" t="str">
         <v>do đó</v>
       </c>
       <c r="K37" t="str">
-        <v>cơn đau đầu</v>
+        <v>dấu hiệu đỏ</v>
       </c>
       <c r="L37" t="str">
-        <v>căng thẳng</v>
+        <v>nghiêm ngặt</v>
       </c>
       <c r="M37" t="str">
         <v/>
@@ -2380,31 +2380,31 @@
         <v>4</v>
       </c>
       <c r="D38" t="str">
-        <v>flight cancellation</v>
+        <v>airport terminal</v>
       </c>
       <c r="E38" t="str">
-        <v>in contrast</v>
+        <v>however</v>
       </c>
       <c r="F38" t="str">
-        <v>dead stop</v>
+        <v>lifeline</v>
       </c>
       <c r="G38" t="str">
-        <v>refunded</v>
+        <v>helpful</v>
       </c>
       <c r="H38" t="str">
         <v/>
       </c>
       <c r="I38" t="str">
-        <v>chuyến bay bị hủy</v>
+        <v>nhà ga sân bay</v>
       </c>
       <c r="J38" t="str">
-        <v>ngược lại</v>
+        <v>tuy nhiên</v>
       </c>
       <c r="K38" t="str">
-        <v>dừng hẳn</v>
+        <v>phao cứu sinh</v>
       </c>
       <c r="L38" t="str">
-        <v>được bồi hoàn</v>
+        <v>hữu ích</v>
       </c>
       <c r="M38" t="str">
         <v/>
@@ -2436,31 +2436,31 @@
         <v>4</v>
       </c>
       <c r="D39" t="str">
-        <v>Why delay</v>
+        <v>Which flight</v>
       </c>
       <c r="E39" t="str">
-        <v>finally</v>
+        <v>otherwise</v>
       </c>
       <c r="F39" t="str">
-        <v>safe harbor</v>
+        <v>last call</v>
       </c>
       <c r="G39" t="str">
-        <v>relieved</v>
+        <v>missed</v>
       </c>
       <c r="H39" t="str">
         <v/>
       </c>
       <c r="I39" t="str">
-        <v>Tại sao lại hoãn</v>
+        <v>Chuyến bay nào</v>
       </c>
       <c r="J39" t="str">
-        <v>sau cùng</v>
+        <v>nếu không</v>
       </c>
       <c r="K39" t="str">
-        <v>bến đỗ an toàn</v>
+        <v>loa gọi chót</v>
       </c>
       <c r="L39" t="str">
-        <v>thở phào</v>
+        <v>lỡ chuyến</v>
       </c>
       <c r="M39" t="str">
         <v/>
@@ -2472,7 +2472,7 @@
         <v>Từ nối · Logic word</v>
       </c>
       <c r="P39" t="str">
-        <v>Ẩn dụ · Fancy word</v>
+        <v>Cụm gợi hình · Fancy word</v>
       </c>
       <c r="Q39" t="str">
         <v>Tính từ · Ending</v>
@@ -2492,31 +2492,31 @@
         <v>4</v>
       </c>
       <c r="D40" t="str">
-        <v>overseas travel</v>
+        <v>flight cancellation</v>
       </c>
       <c r="E40" t="str">
-        <v>as long as</v>
+        <v>eventually</v>
       </c>
       <c r="F40" t="str">
-        <v>Better safe than sorry</v>
+        <v>dead stop</v>
       </c>
       <c r="G40" t="str">
-        <v>prepared</v>
+        <v>refunded</v>
       </c>
       <c r="H40" t="str">
         <v/>
       </c>
       <c r="I40" t="str">
-        <v>du lịch nước ngoài</v>
+        <v>hủy chuyến bay</v>
       </c>
       <c r="J40" t="str">
-        <v>miễn là</v>
+        <v>sau cùng</v>
       </c>
       <c r="K40" t="str">
-        <v>cẩn tắc vô áy náy</v>
+        <v>dừng hẳn</v>
       </c>
       <c r="L40" t="str">
-        <v>chuẩn bị kỹ</v>
+        <v>hoàn tiền</v>
       </c>
       <c r="M40" t="str">
         <v/>
@@ -2528,7 +2528,7 @@
         <v>Từ nối · Logic word</v>
       </c>
       <c r="P40" t="str">
-        <v>Tục ngữ · Proverb</v>
+        <v>Ẩn dụ · Fancy word</v>
       </c>
       <c r="Q40" t="str">
         <v>Tính từ · Ending</v>
@@ -2548,43 +2548,43 @@
         <v>4</v>
       </c>
       <c r="D41" t="str">
-        <v>midnight layover</v>
+        <v>Why delay</v>
       </c>
       <c r="E41" t="str">
-        <v>meanwhile</v>
+        <v>as long as</v>
       </c>
       <c r="F41" t="str">
-        <v>empty chairs</v>
+        <v>safe harbor</v>
       </c>
       <c r="G41" t="str">
-        <v>freezing</v>
+        <v>relieved</v>
       </c>
       <c r="H41" t="str">
         <v/>
       </c>
       <c r="I41" t="str">
-        <v>quá cảnh nửa đêm</v>
+        <v>Sao lại hoãn</v>
       </c>
       <c r="J41" t="str">
-        <v>đồng thời</v>
+        <v>miễn là</v>
       </c>
       <c r="K41" t="str">
-        <v>ghế trống trơn</v>
+        <v>bến đỗ an toàn</v>
       </c>
       <c r="L41" t="str">
-        <v>lạnh cóng</v>
+        <v>thở phào</v>
       </c>
       <c r="M41" t="str">
         <v/>
       </c>
       <c r="N41" t="str">
-        <v>Danh từ · Keyword</v>
+        <v>Cụm nghi vấn · WH word</v>
       </c>
       <c r="O41" t="str">
         <v>Từ nối · Logic word</v>
       </c>
       <c r="P41" t="str">
-        <v>Cụm gợi hình · Fancy word</v>
+        <v>Ẩn dụ · Fancy word</v>
       </c>
       <c r="Q41" t="str">
         <v>Tính từ · Ending</v>
@@ -2604,43 +2604,43 @@
         <v>4</v>
       </c>
       <c r="D42" t="str">
-        <v>How long</v>
+        <v>overseas travel</v>
       </c>
       <c r="E42" t="str">
         <v>if</v>
       </c>
       <c r="F42" t="str">
-        <v>green light</v>
+        <v>Better safe than sorry</v>
       </c>
       <c r="G42" t="str">
-        <v>smooth</v>
+        <v>prepared</v>
       </c>
       <c r="H42" t="str">
         <v/>
       </c>
       <c r="I42" t="str">
-        <v>Bao lâu</v>
+        <v>du lịch nước ngoài</v>
       </c>
       <c r="J42" t="str">
         <v>nếu</v>
       </c>
       <c r="K42" t="str">
-        <v>bật đèn xanh</v>
+        <v>cẩn tắc vô áy náy</v>
       </c>
       <c r="L42" t="str">
-        <v>trơn tru</v>
+        <v>chuẩn bị kỹ</v>
       </c>
       <c r="M42" t="str">
         <v/>
       </c>
       <c r="N42" t="str">
-        <v>Cụm nghi vấn · WH word</v>
+        <v>Danh từ · Keyword</v>
       </c>
       <c r="O42" t="str">
         <v>Từ nối · Logic word</v>
       </c>
       <c r="P42" t="str">
-        <v>Ẩn dụ · Fancy word</v>
+        <v>Tục ngữ · Proverb</v>
       </c>
       <c r="Q42" t="str">
         <v>Tính từ · Ending</v>
@@ -2660,31 +2660,31 @@
         <v>4</v>
       </c>
       <c r="D43" t="str">
-        <v>budget airline</v>
+        <v>midnight layover</v>
       </c>
       <c r="E43" t="str">
-        <v>nevertheless</v>
+        <v>meanwhile</v>
       </c>
       <c r="F43" t="str">
-        <v>hidden cost</v>
+        <v>empty chairs</v>
       </c>
       <c r="G43" t="str">
-        <v>pricey</v>
+        <v>freezing</v>
       </c>
       <c r="H43" t="str">
         <v/>
       </c>
       <c r="I43" t="str">
-        <v>hãng bay giá rẻ</v>
+        <v>quá cảnh nửa đêm</v>
       </c>
       <c r="J43" t="str">
-        <v>dù vậy</v>
+        <v>đồng thời</v>
       </c>
       <c r="K43" t="str">
-        <v>chi phí ngầm</v>
+        <v>ghế trống trơn</v>
       </c>
       <c r="L43" t="str">
-        <v>đắt đỏ</v>
+        <v>lạnh cóng</v>
       </c>
       <c r="M43" t="str">
         <v/>
@@ -2696,7 +2696,7 @@
         <v>Từ nối · Logic word</v>
       </c>
       <c r="P43" t="str">
-        <v>Ẩn dụ · Fancy word</v>
+        <v>Cụm gợi hình · Fancy word</v>
       </c>
       <c r="Q43" t="str">
         <v>Tính từ · Ending</v>
@@ -2716,43 +2716,43 @@
         <v>4</v>
       </c>
       <c r="D44" t="str">
-        <v>commuter train</v>
+        <v>How long</v>
       </c>
       <c r="E44" t="str">
-        <v>before that</v>
+        <v>in addition</v>
       </c>
       <c r="F44" t="str">
-        <v>rush hour</v>
+        <v>green light</v>
       </c>
       <c r="G44" t="str">
-        <v>packed</v>
+        <v>smooth</v>
       </c>
       <c r="H44" t="str">
         <v/>
       </c>
       <c r="I44" t="str">
-        <v>tàu trung chuyển</v>
+        <v>Mất bao lâu</v>
       </c>
       <c r="J44" t="str">
-        <v>trước đó</v>
+        <v>hơn nữa</v>
       </c>
       <c r="K44" t="str">
-        <v>giờ cao điểm</v>
+        <v>bật đèn xanh</v>
       </c>
       <c r="L44" t="str">
-        <v>chật ních</v>
+        <v>trôi chảy</v>
       </c>
       <c r="M44" t="str">
         <v/>
       </c>
       <c r="N44" t="str">
-        <v>Danh từ · Keyword</v>
+        <v>Cụm nghi vấn · WH word</v>
       </c>
       <c r="O44" t="str">
         <v>Từ nối · Logic word</v>
       </c>
       <c r="P44" t="str">
-        <v>Cụm gợi hình · Fancy word</v>
+        <v>Ẩn dụ · Fancy word</v>
       </c>
       <c r="Q44" t="str">
         <v>Tính từ · Ending</v>
@@ -2772,31 +2772,31 @@
         <v>4</v>
       </c>
       <c r="D45" t="str">
-        <v>travel SIM</v>
+        <v>budget airline</v>
       </c>
       <c r="E45" t="str">
-        <v>in addition</v>
+        <v>nevertheless</v>
       </c>
       <c r="F45" t="str">
-        <v>game changer</v>
+        <v>hidden fees</v>
       </c>
       <c r="G45" t="str">
-        <v>connected</v>
+        <v>costly</v>
       </c>
       <c r="H45" t="str">
         <v/>
       </c>
       <c r="I45" t="str">
-        <v>SIM du lịch</v>
+        <v>hãng bay giá rẻ</v>
       </c>
       <c r="J45" t="str">
-        <v>hơn nữa</v>
+        <v>dù vậy</v>
       </c>
       <c r="K45" t="str">
-        <v>bước đột phá</v>
+        <v>chi phí ngầm</v>
       </c>
       <c r="L45" t="str">
-        <v>thông suốt</v>
+        <v>tốn kém</v>
       </c>
       <c r="M45" t="str">
         <v/>
@@ -2828,43 +2828,43 @@
         <v>4</v>
       </c>
       <c r="D46" t="str">
-        <v>Where to go</v>
+        <v>commuter train</v>
       </c>
       <c r="E46" t="str">
-        <v>next</v>
+        <v>before that</v>
       </c>
       <c r="F46" t="str">
-        <v>hidden gem</v>
+        <v>rush hour</v>
       </c>
       <c r="G46" t="str">
-        <v>breathtaking</v>
+        <v>packed</v>
       </c>
       <c r="H46" t="str">
         <v/>
       </c>
       <c r="I46" t="str">
-        <v>Đi đâu bây giờ</v>
+        <v>tàu trung chuyển</v>
       </c>
       <c r="J46" t="str">
-        <v>tiếp theo</v>
+        <v>trước đó</v>
       </c>
       <c r="K46" t="str">
-        <v>viên ngọc ẩn</v>
+        <v>giờ cao điểm</v>
       </c>
       <c r="L46" t="str">
-        <v>tuyệt đẹp</v>
+        <v>chật ních</v>
       </c>
       <c r="M46" t="str">
         <v/>
       </c>
       <c r="N46" t="str">
-        <v>Cụm nghi vấn · WH word</v>
+        <v>Danh từ · Keyword</v>
       </c>
       <c r="O46" t="str">
         <v>Từ nối · Logic word</v>
       </c>
       <c r="P46" t="str">
-        <v>Ẩn dụ · Fancy word</v>
+        <v>Cụm gợi hình · Fancy word</v>
       </c>
       <c r="Q46" t="str">
         <v>Tính từ · Ending</v>
@@ -2884,31 +2884,31 @@
         <v>4</v>
       </c>
       <c r="D47" t="str">
-        <v>emergency exit</v>
+        <v>travel SIM</v>
       </c>
       <c r="E47" t="str">
-        <v>for that reason</v>
+        <v>for example</v>
       </c>
       <c r="F47" t="str">
-        <v>watchful eye</v>
+        <v>game changer</v>
       </c>
       <c r="G47" t="str">
-        <v>alert</v>
+        <v>connected</v>
       </c>
       <c r="H47" t="str">
         <v/>
       </c>
       <c r="I47" t="str">
-        <v>cửa thoát hiểm</v>
+        <v>SIM du lịch</v>
       </c>
       <c r="J47" t="str">
-        <v>chính vì thế</v>
+        <v>ví dụ</v>
       </c>
       <c r="K47" t="str">
-        <v>ánh mắt quan sát</v>
+        <v>bước đột phá</v>
       </c>
       <c r="L47" t="str">
-        <v>cảnh giác</v>
+        <v>thông suốt</v>
       </c>
       <c r="M47" t="str">
         <v/>
@@ -2955,13 +2955,13 @@
         <v/>
       </c>
       <c r="I48" t="str">
-        <v>khu chợ đêm</v>
+        <v>chợ đêm</v>
       </c>
       <c r="J48" t="str">
         <v>sau đó</v>
       </c>
       <c r="K48" t="str">
-        <v>thiên đường món ngon</v>
+        <v>thiên đường ẩm thực</v>
       </c>
       <c r="L48" t="str">
         <v>nhộn nhịp</v>
@@ -2999,31 +2999,31 @@
         <v>Just so you know</v>
       </c>
       <c r="E49" t="str">
-        <v>boarding gate</v>
+        <v>boarding pass</v>
       </c>
       <c r="F49" t="str">
         <v>meanwhile</v>
       </c>
       <c r="G49" t="str">
-        <v>final call</v>
+        <v>smooth sailing</v>
       </c>
       <c r="H49" t="str">
-        <v>hurry</v>
+        <v>on time</v>
       </c>
       <c r="I49" t="str">
-        <v>Nói trước cho bạn hay</v>
+        <v>Nói trước cho bạn biết</v>
       </c>
       <c r="J49" t="str">
-        <v>cửa lên tàu bay</v>
+        <v>thẻ lên máy bay</v>
       </c>
       <c r="K49" t="str">
         <v>đồng thời</v>
       </c>
       <c r="L49" t="str">
-        <v>hiệu lệnh cuối</v>
+        <v>thuận buồm xuôi gió</v>
       </c>
       <c r="M49" t="str">
-        <v>khẩn trương</v>
+        <v>đúng giờ</v>
       </c>
       <c r="N49" t="str">
         <v>Cụm mào đầu · Intro</v>
@@ -3035,10 +3035,10 @@
         <v>Từ nối · Logic word</v>
       </c>
       <c r="Q49" t="str">
-        <v>Cụm gợi hình · Fancy word</v>
+        <v>Ẩn dụ · Fancy word</v>
       </c>
       <c r="R49" t="str">
-        <v>Động từ · Ending</v>
+        <v>Tính từ · Ending</v>
       </c>
     </row>
     <row r="50">
@@ -3052,34 +3052,34 @@
         <v>5</v>
       </c>
       <c r="D50" t="str">
-        <v>To tell you the truth</v>
+        <v>It seems that</v>
       </c>
       <c r="E50" t="str">
-        <v>rough turbulence</v>
+        <v>flight</v>
       </c>
       <c r="F50" t="str">
-        <v>while</v>
+        <v>however</v>
       </c>
       <c r="G50" t="str">
-        <v>roller coaster</v>
+        <v>hectic</v>
       </c>
       <c r="H50" t="str">
-        <v>scary</v>
+        <v>delayed</v>
       </c>
       <c r="I50" t="str">
-        <v>Thật lòng mà nói</v>
+        <v>Hình như là</v>
       </c>
       <c r="J50" t="str">
-        <v>nhiễu động dữ dội</v>
+        <v>chuyến bay</v>
       </c>
       <c r="K50" t="str">
-        <v>trong khi</v>
+        <v>tuy nhiên</v>
       </c>
       <c r="L50" t="str">
-        <v>tàu lượn rung giật</v>
+        <v>nháo nhào</v>
       </c>
       <c r="M50" t="str">
-        <v>đáng sợ</v>
+        <v>hoãn lại</v>
       </c>
       <c r="N50" t="str">
         <v>Cụm mào đầu · Intro</v>
@@ -3091,7 +3091,7 @@
         <v>Từ nối · Logic word</v>
       </c>
       <c r="Q50" t="str">
-        <v>Ẩn dụ · Fancy word</v>
+        <v>Cụm gợi hình · Fancy word</v>
       </c>
       <c r="R50" t="str">
         <v>Tính từ · Ending</v>
@@ -3108,34 +3108,34 @@
         <v>5</v>
       </c>
       <c r="D51" t="str">
-        <v>It seems that</v>
+        <v>To be honest</v>
       </c>
       <c r="E51" t="str">
-        <v>customs officer</v>
+        <v>turbulence</v>
       </c>
       <c r="F51" t="str">
-        <v>however</v>
+        <v>while</v>
       </c>
       <c r="G51" t="str">
-        <v>eagle eye</v>
+        <v>roller coaster</v>
       </c>
       <c r="H51" t="str">
-        <v>thorough</v>
+        <v>scary</v>
       </c>
       <c r="I51" t="str">
-        <v>Có vẻ như là</v>
+        <v>Thành thật mà nói</v>
       </c>
       <c r="J51" t="str">
-        <v>nhân viên hải quan</v>
+        <v>nhiễu động không khí</v>
       </c>
       <c r="K51" t="str">
-        <v>tuy nhiên</v>
+        <v>trong khi</v>
       </c>
       <c r="L51" t="str">
-        <v>mắt đại bàng</v>
+        <v>tàu lượn</v>
       </c>
       <c r="M51" t="str">
-        <v>kỹ lưỡng</v>
+        <v>đáng sợ</v>
       </c>
       <c r="N51" t="str">
         <v>Cụm mào đầu · Intro</v>
@@ -3167,31 +3167,31 @@
         <v>As far as I know</v>
       </c>
       <c r="E52" t="str">
-        <v>entry visa</v>
+        <v>customs officer</v>
       </c>
       <c r="F52" t="str">
-        <v>otherwise</v>
+        <v>therefore</v>
       </c>
       <c r="G52" t="str">
-        <v>red tape</v>
+        <v>eagle eye</v>
       </c>
       <c r="H52" t="str">
-        <v>delayed</v>
+        <v>strict</v>
       </c>
       <c r="I52" t="str">
         <v>Theo chỗ tôi biết</v>
       </c>
       <c r="J52" t="str">
-        <v>thị thực nhập cảnh</v>
+        <v>nhân viên hải quan</v>
       </c>
       <c r="K52" t="str">
-        <v>nếu không</v>
+        <v>do đó</v>
       </c>
       <c r="L52" t="str">
-        <v>thủ tục quan liêu</v>
+        <v>mắt đại bàng</v>
       </c>
       <c r="M52" t="str">
-        <v>bị ách lại</v>
+        <v>nghiêm ngặt</v>
       </c>
       <c r="N52" t="str">
         <v>Cụm mào đầu · Intro</v>
@@ -3223,31 +3223,31 @@
         <v>Believe it or not</v>
       </c>
       <c r="E53" t="str">
-        <v>baggage carousel</v>
+        <v>entry visa</v>
       </c>
       <c r="F53" t="str">
-        <v>eventually</v>
+        <v>otherwise</v>
       </c>
       <c r="G53" t="str">
-        <v>dead end</v>
+        <v>red tape</v>
       </c>
       <c r="H53" t="str">
-        <v>jammed</v>
+        <v>rejected</v>
       </c>
       <c r="I53" t="str">
         <v>Tin hay không tùy bạn</v>
       </c>
       <c r="J53" t="str">
-        <v>băng chuyền hành lý</v>
+        <v>thị thực nhập cảnh</v>
       </c>
       <c r="K53" t="str">
-        <v>sau cùng</v>
+        <v>nếu không</v>
       </c>
       <c r="L53" t="str">
-        <v>chỗ kẹt nghẽn</v>
+        <v>thủ tục quan liêu</v>
       </c>
       <c r="M53" t="str">
-        <v>bị kẹt cứng</v>
+        <v>bị từ chối</v>
       </c>
       <c r="N53" t="str">
         <v>Cụm mào đầu · Intro</v>
@@ -3276,34 +3276,34 @@
         <v>5</v>
       </c>
       <c r="D54" t="str">
-        <v>From my perspective</v>
+        <v>From my experience</v>
       </c>
       <c r="E54" t="str">
-        <v>sleeping pod</v>
+        <v>baggage claim</v>
       </c>
       <c r="F54" t="str">
-        <v>in addition</v>
+        <v>eventually</v>
       </c>
       <c r="G54" t="str">
-        <v>godsend</v>
+        <v>bottleneck</v>
       </c>
       <c r="H54" t="str">
-        <v>comfortable</v>
+        <v>crowded</v>
       </c>
       <c r="I54" t="str">
-        <v>Theo góc nhìn của tôi</v>
+        <v>Theo kinh nghiệm của tôi</v>
       </c>
       <c r="J54" t="str">
-        <v>buồng ngủ sân bay</v>
+        <v>nhận hành lý</v>
       </c>
       <c r="K54" t="str">
-        <v>hơn nữa</v>
+        <v>sau cùng</v>
       </c>
       <c r="L54" t="str">
-        <v>món quà cứu cánh</v>
+        <v>nút thắt cổ chai</v>
       </c>
       <c r="M54" t="str">
-        <v>dễ chịu</v>
+        <v>đông đúc</v>
       </c>
       <c r="N54" t="str">
         <v>Cụm mào đầu · Intro</v>
@@ -3335,31 +3335,31 @@
         <v>In my opinion</v>
       </c>
       <c r="E55" t="str">
-        <v>street food</v>
+        <v>sleeping pod</v>
       </c>
       <c r="F55" t="str">
-        <v>if</v>
+        <v>in addition</v>
       </c>
       <c r="G55" t="str">
-        <v>gold mine</v>
+        <v>lifesaver</v>
       </c>
       <c r="H55" t="str">
-        <v>authentic</v>
+        <v>cozy</v>
       </c>
       <c r="I55" t="str">
         <v>Theo quan điểm của tôi</v>
       </c>
       <c r="J55" t="str">
-        <v>món ăn đường phố</v>
+        <v>buồng ngủ mini</v>
       </c>
       <c r="K55" t="str">
-        <v>nếu</v>
+        <v>hơn nữa</v>
       </c>
       <c r="L55" t="str">
-        <v>mỏ vàng ẩm thực</v>
+        <v>vị cứu tinh</v>
       </c>
       <c r="M55" t="str">
-        <v>chuẩn vị</v>
+        <v>ấm cúng</v>
       </c>
       <c r="N55" t="str">
         <v>Cụm mào đầu · Intro</v>
@@ -3391,31 +3391,31 @@
         <v>Don't get me wrong</v>
       </c>
       <c r="E56" t="str">
-        <v>souvenir shop</v>
+        <v>street food</v>
       </c>
       <c r="F56" t="str">
-        <v>nevertheless</v>
+        <v>if</v>
       </c>
       <c r="G56" t="str">
-        <v>tourist trap</v>
+        <v>gold mine</v>
       </c>
       <c r="H56" t="str">
-        <v>pricey</v>
+        <v>delicious</v>
       </c>
       <c r="I56" t="str">
         <v>Đừng hiểu sai ý tôi</v>
       </c>
       <c r="J56" t="str">
-        <v>cửa hàng lưu niệm</v>
+        <v>món ăn đường phố</v>
       </c>
       <c r="K56" t="str">
-        <v>dù vậy</v>
+        <v>nếu</v>
       </c>
       <c r="L56" t="str">
-        <v>cái bẫy du khách</v>
+        <v>mỏ vàng</v>
       </c>
       <c r="M56" t="str">
-        <v>đắt đỏ</v>
+        <v>ngon tuyệt</v>
       </c>
       <c r="N56" t="str">
         <v>Cụm mào đầu · Intro</v>
@@ -3447,31 +3447,31 @@
         <v>As a matter of fact</v>
       </c>
       <c r="E57" t="str">
-        <v>flight attendant</v>
+        <v>souvenir shop</v>
       </c>
       <c r="F57" t="str">
-        <v>therefore</v>
+        <v>nevertheless</v>
       </c>
       <c r="G57" t="str">
-        <v>lifesaver</v>
+        <v>tourist trap</v>
       </c>
       <c r="H57" t="str">
-        <v>supportive</v>
+        <v>overpriced</v>
       </c>
       <c r="I57" t="str">
         <v>Thực tế là</v>
       </c>
       <c r="J57" t="str">
-        <v>tiếp viên hàng không</v>
+        <v>cửa hàng lưu niệm</v>
       </c>
       <c r="K57" t="str">
-        <v>do đó</v>
+        <v>dù vậy</v>
       </c>
       <c r="L57" t="str">
-        <v>vị cứu tinh</v>
+        <v>cái bẫy du khách</v>
       </c>
       <c r="M57" t="str">
-        <v>tận tình</v>
+        <v>quá đắt</v>
       </c>
       <c r="N57" t="str">
         <v>Cụm mào đầu · Intro</v>
@@ -3503,7 +3503,7 @@
         <v>First of all</v>
       </c>
       <c r="E58" t="str">
-        <v>medical insurance</v>
+        <v>travel insurance</v>
       </c>
       <c r="F58" t="str">
         <v>before that</v>
@@ -3518,13 +3518,13 @@
         <v>Trước hết là</v>
       </c>
       <c r="J58" t="str">
-        <v>bảo hiểm y tế</v>
+        <v>bảo hiểm du lịch</v>
       </c>
       <c r="K58" t="str">
         <v>trước đó</v>
       </c>
       <c r="L58" t="str">
-        <v>lưới bảo hiểm an toàn</v>
+        <v>lưới an toàn</v>
       </c>
       <c r="M58" t="str">
         <v>sống còn</v>
@@ -3559,31 +3559,31 @@
         <v>By the way</v>
       </c>
       <c r="E59" t="str">
-        <v>hotel reception</v>
+        <v>flight attendant</v>
       </c>
       <c r="F59" t="str">
-        <v>next</v>
+        <v>in other words</v>
       </c>
       <c r="G59" t="str">
-        <v>warm welcome</v>
+        <v>helping hand</v>
       </c>
       <c r="H59" t="str">
-        <v>hospitable</v>
+        <v>supportive</v>
       </c>
       <c r="I59" t="str">
         <v>Nhân tiện đây</v>
       </c>
       <c r="J59" t="str">
-        <v>tiếp tân khách sạn</v>
+        <v>tiếp viên hàng không</v>
       </c>
       <c r="K59" t="str">
-        <v>tiếp theo</v>
+        <v>nói cách khác</v>
       </c>
       <c r="L59" t="str">
-        <v>chào đón ấm áp</v>
+        <v>bàn tay tương trợ</v>
       </c>
       <c r="M59" t="str">
-        <v>hiếu khách</v>
+        <v>tận tình</v>
       </c>
       <c r="N59" t="str">
         <v>Cụm mào đầu · Intro</v>
@@ -3595,7 +3595,7 @@
         <v>Từ nối · Logic word</v>
       </c>
       <c r="Q59" t="str">
-        <v>Cụm gợi hình · Fancy word</v>
+        <v>Ẩn dụ · Fancy word</v>
       </c>
       <c r="R59" t="str">
         <v>Tính từ · Ending</v>
@@ -3612,34 +3612,34 @@
         <v>5</v>
       </c>
       <c r="D60" t="str">
-        <v>Honestly speaking</v>
+        <v>Truth be told</v>
       </c>
       <c r="E60" t="str">
-        <v>overweight luggage</v>
+        <v>hotel reception</v>
       </c>
       <c r="F60" t="str">
-        <v>in other words</v>
+        <v>next</v>
       </c>
       <c r="G60" t="str">
-        <v>money pit</v>
+        <v>warm welcome</v>
       </c>
       <c r="H60" t="str">
-        <v>costly</v>
+        <v>friendly</v>
       </c>
       <c r="I60" t="str">
-        <v>Thành thật mà nói</v>
+        <v>Nói thật lòng</v>
       </c>
       <c r="J60" t="str">
-        <v>hành lý quá cước</v>
+        <v>tiếp tân khách sạn</v>
       </c>
       <c r="K60" t="str">
-        <v>nói cách khác</v>
+        <v>tiếp theo</v>
       </c>
       <c r="L60" t="str">
-        <v>hố ngốn tiền</v>
+        <v>chào đón ấm áp</v>
       </c>
       <c r="M60" t="str">
-        <v>hao tốn</v>
+        <v>thân thiện</v>
       </c>
       <c r="N60" t="str">
         <v>Cụm mào đầu · Intro</v>
@@ -3651,7 +3651,7 @@
         <v>Từ nối · Logic word</v>
       </c>
       <c r="Q60" t="str">
-        <v>Ẩn dụ · Fancy word</v>
+        <v>Cụm gợi hình · Fancy word</v>
       </c>
       <c r="R60" t="str">
         <v>Tính từ · Ending</v>
@@ -3668,34 +3668,34 @@
         <v>5</v>
       </c>
       <c r="D61" t="str">
-        <v>Keep in mind</v>
+        <v>Strictly speaking</v>
       </c>
       <c r="E61" t="str">
-        <v>meter taxi</v>
+        <v>overweight luggage</v>
       </c>
       <c r="F61" t="str">
         <v>as long as</v>
       </c>
       <c r="G61" t="str">
-        <v>fair play</v>
+        <v>wake-up call</v>
       </c>
       <c r="H61" t="str">
-        <v>honest</v>
+        <v>avoidable</v>
       </c>
       <c r="I61" t="str">
-        <v>Hãy luôn ghi nhớ</v>
+        <v>Nói nghiêm túc</v>
       </c>
       <c r="J61" t="str">
-        <v>taxi có đồng hồ</v>
+        <v>hành lý quá cước</v>
       </c>
       <c r="K61" t="str">
         <v>miễn là</v>
       </c>
       <c r="L61" t="str">
-        <v>chơi đẹp minh bạch</v>
+        <v>lời cảnh tỉnh</v>
       </c>
       <c r="M61" t="str">
-        <v>trung thực</v>
+        <v>tránh được</v>
       </c>
       <c r="N61" t="str">
         <v>Cụm mào đầu · Intro</v>
@@ -3724,34 +3724,34 @@
         <v>5</v>
       </c>
       <c r="D62" t="str">
-        <v>You can bet that</v>
+        <v>You should know</v>
       </c>
       <c r="E62" t="str">
-        <v>ocean sunrise</v>
+        <v>boarding gate</v>
       </c>
       <c r="F62" t="str">
         <v>then</v>
       </c>
       <c r="G62" t="str">
-        <v>postcard view</v>
+        <v>final call</v>
       </c>
       <c r="H62" t="str">
-        <v>stunning</v>
+        <v>hurry</v>
       </c>
       <c r="I62" t="str">
-        <v>Bạn cứ yên tâm rằng</v>
+        <v>Bạn nên biết</v>
       </c>
       <c r="J62" t="str">
-        <v>bình minh biển</v>
+        <v>cửa khởi hành</v>
       </c>
       <c r="K62" t="str">
         <v>sau đó</v>
       </c>
       <c r="L62" t="str">
-        <v>khung cảnh như tranh</v>
+        <v>hiệu lệnh cuối</v>
       </c>
       <c r="M62" t="str">
-        <v>đẹp ngỡ ngàng</v>
+        <v>khẩn trương</v>
       </c>
       <c r="N62" t="str">
         <v>Cụm mào đầu · Intro</v>
@@ -3766,7 +3766,7 @@
         <v>Cụm gợi hình · Fancy word</v>
       </c>
       <c r="R62" t="str">
-        <v>Tính từ · Ending</v>
+        <v>Động từ · Ending</v>
       </c>
     </row>
     <row r="63">
@@ -3780,34 +3780,34 @@
         <v>5</v>
       </c>
       <c r="D63" t="str">
-        <v>All things considered</v>
+        <v>At the same time</v>
       </c>
       <c r="E63" t="str">
-        <v>solo trip</v>
+        <v>taxi driver</v>
       </c>
       <c r="F63" t="str">
-        <v>finally</v>
+        <v>besides</v>
       </c>
       <c r="G63" t="str">
-        <v>eye opener</v>
+        <v>local guide</v>
       </c>
       <c r="H63" t="str">
-        <v>unforgettable</v>
+        <v>reliable</v>
       </c>
       <c r="I63" t="str">
-        <v>Cân nhắc mọi mặt</v>
+        <v>Đồng thời</v>
       </c>
       <c r="J63" t="str">
-        <v>chuyến du hành độc hành</v>
+        <v>tài xế taxi</v>
       </c>
       <c r="K63" t="str">
-        <v>cuối cùng</v>
+        <v>ngoài ra</v>
       </c>
       <c r="L63" t="str">
-        <v>trải nghiệm mở rộng tầm mắt</v>
+        <v>chỉ dẫn bản địa</v>
       </c>
       <c r="M63" t="str">
-        <v>khó quên</v>
+        <v>đáng tin</v>
       </c>
       <c r="N63" t="str">
         <v>Cụm mào đầu · Intro</v>

</xml_diff>